<commit_message>
feat: Logit-space share convergence + ENLONG alpha harmonization
Share indicators now use Logit-space convergence for all 3 methods:
- Kaya: L_c(t) = L_c(2015) + phi_Kaya(t) * delta_L_R(t)
- DSCALE: ENSHORT/ENLONG dual-path in Logit space
- Logit: Full delta_L_R superposition (unchanged)
All shares now bounded to [0,1] (was: Kaya/DSCALE had 46/35 countries >1.0,
with NZL green_elec 240%, UAE 310%).

DSCALE: Added missing ENLONG alpha harmonization (official
fun_harmonize_alpha at enlong_calc_2021:22944). Base year 2015.

CLAUDE.md: Revised Kaya method description with literature comparison
table (van Vuuren 2007 vs our implementation). Corrected Grubler 1991
citation (wrong title/pages). Added Gutschow 2021 SSP convergence ref.
Refined "original method" claims for academic precision.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compare/output/dscale_Elec_downscaled_SSP126.xlsx
+++ b/compare/output/dscale_Elec_downscaled_SSP126.xlsx
@@ -526,19 +526,19 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3973.788721</v>
+        <v>3975.380044</v>
       </c>
       <c r="F2" t="n">
-        <v>9779.972656</v>
+        <v>9789.859775999999</v>
       </c>
       <c r="G2" t="n">
-        <v>19990.375025</v>
+        <v>20030.847755</v>
       </c>
       <c r="H2" t="n">
-        <v>36759.501579</v>
+        <v>36908.250319</v>
       </c>
       <c r="I2" t="n">
-        <v>63506.749658</v>
+        <v>64144.453076</v>
       </c>
       <c r="J2" t="n">
         <v>44036.095355</v>
@@ -602,19 +602,19 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>335.491343</v>
+        <v>335.505645</v>
       </c>
       <c r="F3" t="n">
-        <v>733.515689</v>
+        <v>733.597978</v>
       </c>
       <c r="G3" t="n">
-        <v>1412.622351</v>
+        <v>1412.921577</v>
       </c>
       <c r="H3" t="n">
-        <v>2574.046389</v>
+        <v>2575.055029</v>
       </c>
       <c r="I3" t="n">
-        <v>4526.299228</v>
+        <v>4530.381284</v>
       </c>
       <c r="J3" t="n">
         <v>7407.211217</v>
@@ -678,19 +678,19 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>399.837328</v>
+        <v>399.554421</v>
       </c>
       <c r="F4" t="n">
-        <v>753.601049</v>
+        <v>752.285744</v>
       </c>
       <c r="G4" t="n">
-        <v>1229.930361</v>
+        <v>1225.673623</v>
       </c>
       <c r="H4" t="n">
-        <v>1996.086119</v>
+        <v>1982.395644</v>
       </c>
       <c r="I4" t="n">
-        <v>3278.952452</v>
+        <v>3224.519703</v>
       </c>
       <c r="J4" t="n">
         <v>10347.327034</v>
@@ -754,19 +754,19 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1044.562585</v>
+        <v>1044.230173</v>
       </c>
       <c r="F5" t="n">
-        <v>2873.056918</v>
+        <v>2870.7089</v>
       </c>
       <c r="G5" t="n">
-        <v>7256.207594</v>
+        <v>7243.760512</v>
       </c>
       <c r="H5" t="n">
-        <v>16128.015908</v>
+        <v>16070.806814</v>
       </c>
       <c r="I5" t="n">
-        <v>32003.257588</v>
+        <v>31720.027492</v>
       </c>
       <c r="J5" t="n">
         <v>87017.987675</v>
@@ -830,19 +830,19 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>38162.561315</v>
+        <v>38164.303446</v>
       </c>
       <c r="F6" t="n">
-        <v>91492.034852</v>
+        <v>91502.538709</v>
       </c>
       <c r="G6" t="n">
-        <v>166872.036214</v>
+        <v>166910.492943</v>
       </c>
       <c r="H6" t="n">
-        <v>280086.910512</v>
+        <v>280216.420047</v>
       </c>
       <c r="I6" t="n">
-        <v>463375.640445</v>
+        <v>463903.064117</v>
       </c>
       <c r="J6" t="n">
         <v>709165.09003</v>
@@ -906,19 +906,19 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>35533.932454</v>
+        <v>35540.393542</v>
       </c>
       <c r="F7" t="n">
-        <v>88480.75834299999</v>
+        <v>88521.140697</v>
       </c>
       <c r="G7" t="n">
-        <v>192995.67673</v>
+        <v>193168.26885</v>
       </c>
       <c r="H7" t="n">
-        <v>390774.334482</v>
+        <v>391455.990503</v>
       </c>
       <c r="I7" t="n">
-        <v>741029.948297</v>
+        <v>744162.8673780001</v>
       </c>
       <c r="J7" t="n">
         <v>1004218.898752</v>
@@ -982,19 +982,19 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>7724.647009</v>
+        <v>7724.453763</v>
       </c>
       <c r="F8" t="n">
-        <v>18456.355578</v>
+        <v>18455.206022</v>
       </c>
       <c r="G8" t="n">
-        <v>37010.619229</v>
+        <v>37005.440976</v>
       </c>
       <c r="H8" t="n">
-        <v>67705.067486</v>
+        <v>67684.479578</v>
       </c>
       <c r="I8" t="n">
-        <v>118276.227387</v>
+        <v>118183.192509</v>
       </c>
       <c r="J8" t="n">
         <v>208224.124501</v>
@@ -1058,19 +1058,19 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10935.183565</v>
+        <v>10938.401972</v>
       </c>
       <c r="F9" t="n">
-        <v>20102.386026</v>
+        <v>20117.499911</v>
       </c>
       <c r="G9" t="n">
-        <v>30525.535749</v>
+        <v>30571.970961</v>
       </c>
       <c r="H9" t="n">
-        <v>44566.797191</v>
+        <v>44703.278229</v>
       </c>
       <c r="I9" t="n">
-        <v>64655.535839</v>
+        <v>65148.678211</v>
       </c>
       <c r="J9" t="n">
         <v>52420.368149</v>
@@ -1134,19 +1134,19 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1928.457112</v>
+        <v>1925.559231</v>
       </c>
       <c r="F10" t="n">
-        <v>4325.05</v>
+        <v>4308.803472</v>
       </c>
       <c r="G10" t="n">
-        <v>7791.853589</v>
+        <v>7733.596917</v>
       </c>
       <c r="H10" t="n">
-        <v>13342.774665</v>
+        <v>13145.984921</v>
       </c>
       <c r="I10" t="n">
-        <v>22958.027829</v>
+        <v>22153.520363</v>
       </c>
       <c r="J10" t="n">
         <v>115396.538831</v>
@@ -1210,19 +1210,19 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>47685.592638</v>
+        <v>47681.147748</v>
       </c>
       <c r="F11" t="n">
-        <v>110358.53254</v>
+        <v>110332.87596</v>
       </c>
       <c r="G11" t="n">
-        <v>215558.166294</v>
+        <v>215454.646793</v>
       </c>
       <c r="H11" t="n">
-        <v>391782.600784</v>
+        <v>391395.648461</v>
       </c>
       <c r="I11" t="n">
-        <v>678568.376064</v>
+        <v>676892.991559</v>
       </c>
       <c r="J11" t="n">
         <v>1236583.163539</v>
@@ -1286,19 +1286,19 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4221.16516</v>
+        <v>4222.601105</v>
       </c>
       <c r="F12" t="n">
-        <v>10201.101625</v>
+        <v>10209.847283</v>
       </c>
       <c r="G12" t="n">
-        <v>21265.559222</v>
+        <v>21301.903296</v>
       </c>
       <c r="H12" t="n">
-        <v>40738.140982</v>
+        <v>40876.582865</v>
       </c>
       <c r="I12" t="n">
-        <v>72921.973708</v>
+        <v>73533.686661</v>
       </c>
       <c r="J12" t="n">
         <v>64628.198996</v>
@@ -1362,19 +1362,19 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>13075.112771</v>
+        <v>13068.800908</v>
       </c>
       <c r="F13" t="n">
-        <v>31348.869025</v>
+        <v>31310.869849</v>
       </c>
       <c r="G13" t="n">
-        <v>61889.639442</v>
+        <v>61738.697597</v>
       </c>
       <c r="H13" t="n">
-        <v>114847.099505</v>
+        <v>114286.483188</v>
       </c>
       <c r="I13" t="n">
-        <v>209186.925105</v>
+        <v>206690.531246</v>
       </c>
       <c r="J13" t="n">
         <v>624999.427521</v>
@@ -1438,19 +1438,19 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>246598.466803</v>
+        <v>246593.312619</v>
       </c>
       <c r="F14" t="n">
-        <v>311381.637681</v>
+        <v>311364.371531</v>
       </c>
       <c r="G14" t="n">
-        <v>403811.838302</v>
+        <v>403766.94954</v>
       </c>
       <c r="H14" t="n">
-        <v>530291.634496</v>
+        <v>530176.771135</v>
       </c>
       <c r="I14" t="n">
-        <v>693539.792175</v>
+        <v>693187.384162</v>
       </c>
       <c r="J14" t="n">
         <v>981501.19978</v>
@@ -1514,19 +1514,19 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>667062.200406</v>
+        <v>667076.062053</v>
       </c>
       <c r="F15" t="n">
-        <v>924227.8717810001</v>
+        <v>924275.96772</v>
       </c>
       <c r="G15" t="n">
-        <v>1250718.464032</v>
+        <v>1250846.230136</v>
       </c>
       <c r="H15" t="n">
-        <v>1672371.552515</v>
+        <v>1672699.586231</v>
       </c>
       <c r="I15" t="n">
-        <v>2191244.766935</v>
+        <v>2192246.973245</v>
       </c>
       <c r="J15" t="n">
         <v>2409049.763831</v>
@@ -1590,19 +1590,19 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>134412.014387</v>
+        <v>134414.069878</v>
       </c>
       <c r="F16" t="n">
-        <v>145789.2406</v>
+        <v>145792.676068</v>
       </c>
       <c r="G16" t="n">
-        <v>156708.905493</v>
+        <v>156711.851244</v>
       </c>
       <c r="H16" t="n">
-        <v>177150.353987</v>
+        <v>177149.531325</v>
       </c>
       <c r="I16" t="n">
-        <v>208775.16902</v>
+        <v>208758.963977</v>
       </c>
       <c r="J16" t="n">
         <v>252624.347839</v>
@@ -1666,19 +1666,19 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>110511.378128</v>
+        <v>110503.922255</v>
       </c>
       <c r="F17" t="n">
-        <v>143022.59552</v>
+        <v>142998.969359</v>
       </c>
       <c r="G17" t="n">
-        <v>183496.193915</v>
+        <v>183437.027067</v>
       </c>
       <c r="H17" t="n">
-        <v>234386.902736</v>
+        <v>234240.521071</v>
       </c>
       <c r="I17" t="n">
-        <v>298029.246008</v>
+        <v>297593.022088</v>
       </c>
       <c r="J17" t="n">
         <v>498403.606651</v>
@@ -1742,19 +1742,19 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>70523.980211</v>
+        <v>70520.673131</v>
       </c>
       <c r="F18" t="n">
-        <v>93572.85677699999</v>
+        <v>93562.217683</v>
       </c>
       <c r="G18" t="n">
-        <v>116195.767758</v>
+        <v>116169.111512</v>
       </c>
       <c r="H18" t="n">
-        <v>143658.529965</v>
+        <v>143592.563938</v>
       </c>
       <c r="I18" t="n">
-        <v>179819.043562</v>
+        <v>179621.674228</v>
       </c>
       <c r="J18" t="n">
         <v>284361.9756</v>
@@ -1818,19 +1818,19 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>36577.915882</v>
+        <v>36566.132985</v>
       </c>
       <c r="F19" t="n">
-        <v>61319.415806</v>
+        <v>61270.568226</v>
       </c>
       <c r="G19" t="n">
-        <v>80151.08268399999</v>
+        <v>80022.28148799999</v>
       </c>
       <c r="H19" t="n">
-        <v>118448.282861</v>
+        <v>118062.754931</v>
       </c>
       <c r="I19" t="n">
-        <v>179847.607483</v>
+        <v>178392.928069</v>
       </c>
       <c r="J19" t="n">
         <v>712910.717817</v>
@@ -1894,19 +1894,19 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>10655.247774</v>
+        <v>10653.940652</v>
       </c>
       <c r="F20" t="n">
-        <v>16303.04013</v>
+        <v>16298.119827</v>
       </c>
       <c r="G20" t="n">
-        <v>21094.807294</v>
+        <v>21081.627222</v>
       </c>
       <c r="H20" t="n">
-        <v>30733.098414</v>
+        <v>30692.603344</v>
       </c>
       <c r="I20" t="n">
-        <v>44532.711749</v>
+        <v>44379.907511</v>
       </c>
       <c r="J20" t="n">
         <v>106468.484108</v>
@@ -1970,19 +1970,19 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>965.658409</v>
+        <v>965.315867</v>
       </c>
       <c r="F21" t="n">
-        <v>1305.04004</v>
+        <v>1303.890634</v>
       </c>
       <c r="G21" t="n">
-        <v>1497.492109</v>
+        <v>1494.832299</v>
       </c>
       <c r="H21" t="n">
-        <v>2092.223183</v>
+        <v>2084.72086</v>
       </c>
       <c r="I21" t="n">
-        <v>3127.186392</v>
+        <v>3099.462876</v>
       </c>
       <c r="J21" t="n">
         <v>13081.100311</v>
@@ -2046,19 +2046,19 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>69609.707224</v>
+        <v>69620.913529</v>
       </c>
       <c r="F22" t="n">
-        <v>117405.964157</v>
+        <v>117453.420923</v>
       </c>
       <c r="G22" t="n">
-        <v>154266.219324</v>
+        <v>154386.184245</v>
       </c>
       <c r="H22" t="n">
-        <v>226730.505542</v>
+        <v>227061.881869</v>
       </c>
       <c r="I22" t="n">
-        <v>337241.741728</v>
+        <v>338383.832816</v>
       </c>
       <c r="J22" t="n">
         <v>172567.68582</v>
@@ -2122,19 +2122,19 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>7315.638602</v>
+        <v>7314.869361</v>
       </c>
       <c r="F23" t="n">
-        <v>12781.348909</v>
+        <v>12778.057641</v>
       </c>
       <c r="G23" t="n">
-        <v>17924.811531</v>
+        <v>17915.187254</v>
       </c>
       <c r="H23" t="n">
-        <v>28856.549559</v>
+        <v>28823.573469</v>
       </c>
       <c r="I23" t="n">
-        <v>47324.378696</v>
+        <v>47182.405901</v>
       </c>
       <c r="J23" t="n">
         <v>124725.7559</v>
@@ -2198,19 +2198,19 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>5832.668513</v>
+        <v>5831.662062</v>
       </c>
       <c r="F24" t="n">
-        <v>8991.841923</v>
+        <v>8988.012631</v>
       </c>
       <c r="G24" t="n">
-        <v>11394.594604</v>
+        <v>11384.659943</v>
       </c>
       <c r="H24" t="n">
-        <v>16495.192335</v>
+        <v>16465.397256</v>
       </c>
       <c r="I24" t="n">
-        <v>24168.268847</v>
+        <v>24056.781334</v>
       </c>
       <c r="J24" t="n">
         <v>67575.695288</v>
@@ -2274,19 +2274,19 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1430.703235</v>
+        <v>1430.204661</v>
       </c>
       <c r="F25" t="n">
-        <v>2052.989181</v>
+        <v>2051.215255</v>
       </c>
       <c r="G25" t="n">
-        <v>2522.621765</v>
+        <v>2518.231654</v>
       </c>
       <c r="H25" t="n">
-        <v>3707.187245</v>
+        <v>3694.169594</v>
       </c>
       <c r="I25" t="n">
-        <v>5596.765215</v>
+        <v>5548.137159</v>
       </c>
       <c r="J25" t="n">
         <v>22650.58683</v>
@@ -2350,19 +2350,19 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>24616.186873</v>
+        <v>24607.422494</v>
       </c>
       <c r="F26" t="n">
-        <v>40473.5587</v>
+        <v>40437.90906</v>
       </c>
       <c r="G26" t="n">
-        <v>50317.85646</v>
+        <v>50228.51373</v>
       </c>
       <c r="H26" t="n">
-        <v>70119.37611899999</v>
+        <v>69867.582142</v>
       </c>
       <c r="I26" t="n">
-        <v>101441.752869</v>
+        <v>100539.039689</v>
       </c>
       <c r="J26" t="n">
         <v>413177.466588</v>
@@ -2426,19 +2426,19 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>50777.509311</v>
+        <v>50782.670137</v>
       </c>
       <c r="F27" t="n">
-        <v>83970.620549</v>
+        <v>83992.141947</v>
       </c>
       <c r="G27" t="n">
-        <v>107382.293708</v>
+        <v>107434.12349</v>
       </c>
       <c r="H27" t="n">
-        <v>157835.50541</v>
+        <v>157973.494171</v>
       </c>
       <c r="I27" t="n">
-        <v>237633.037509</v>
+        <v>238091.952075</v>
       </c>
       <c r="J27" t="n">
         <v>230338.137193</v>
@@ -2502,19 +2502,19 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>36500.208477</v>
+        <v>36508.31255</v>
       </c>
       <c r="F28" t="n">
-        <v>54811.851419</v>
+        <v>54842.334671</v>
       </c>
       <c r="G28" t="n">
-        <v>79722.26206199999</v>
+        <v>79808.40021599999</v>
       </c>
       <c r="H28" t="n">
-        <v>141255.483942</v>
+        <v>141547.226974</v>
       </c>
       <c r="I28" t="n">
-        <v>253325.544122</v>
+        <v>254564.547181</v>
       </c>
       <c r="J28" t="n">
         <v>19595.687754</v>
@@ -2578,19 +2578,19 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1001.524757</v>
+        <v>1001.360281</v>
       </c>
       <c r="F29" t="n">
-        <v>1470.975427</v>
+        <v>1470.36075</v>
       </c>
       <c r="G29" t="n">
-        <v>2204.506709</v>
+        <v>2202.59037</v>
       </c>
       <c r="H29" t="n">
-        <v>3619.277822</v>
+        <v>3612.726045</v>
       </c>
       <c r="I29" t="n">
-        <v>6070.933326</v>
+        <v>6042.609378</v>
       </c>
       <c r="J29" t="n">
         <v>43462.996491</v>
@@ -2654,19 +2654,19 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>5739.428384</v>
+        <v>5739.447761</v>
       </c>
       <c r="F30" t="n">
-        <v>7962.082222</v>
+        <v>7962.167332</v>
       </c>
       <c r="G30" t="n">
-        <v>11236.148134</v>
+        <v>11236.31518</v>
       </c>
       <c r="H30" t="n">
-        <v>17851.010285</v>
+        <v>17851.234091</v>
       </c>
       <c r="I30" t="n">
-        <v>28867.660739</v>
+        <v>28867.745118</v>
       </c>
       <c r="J30" t="n">
         <v>46994.530528</v>
@@ -2730,19 +2730,19 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1645.864322</v>
+        <v>1645.893513</v>
       </c>
       <c r="F31" t="n">
-        <v>2548.162909</v>
+        <v>2548.276271</v>
       </c>
       <c r="G31" t="n">
-        <v>3831.097865</v>
+        <v>3831.405542</v>
       </c>
       <c r="H31" t="n">
-        <v>6298.404805</v>
+        <v>6299.298695</v>
       </c>
       <c r="I31" t="n">
-        <v>10497.609032</v>
+        <v>10500.995455</v>
       </c>
       <c r="J31" t="n">
         <v>13542.250326</v>
@@ -2806,19 +2806,19 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>26422.784399</v>
+        <v>26423.690832</v>
       </c>
       <c r="F32" t="n">
-        <v>35509.735773</v>
+        <v>35512.883903</v>
       </c>
       <c r="G32" t="n">
-        <v>48900.412364</v>
+        <v>48908.884876</v>
       </c>
       <c r="H32" t="n">
-        <v>76571.02617</v>
+        <v>76596.77587899999</v>
       </c>
       <c r="I32" t="n">
-        <v>125307.81761</v>
+        <v>125411.50518</v>
       </c>
       <c r="J32" t="n">
         <v>86607.804691</v>
@@ -2882,19 +2882,19 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>24191.254511</v>
+        <v>24191.737407</v>
       </c>
       <c r="F33" t="n">
-        <v>35238.534154</v>
+        <v>35240.341268</v>
       </c>
       <c r="G33" t="n">
-        <v>52324.270301</v>
+        <v>52329.230898</v>
       </c>
       <c r="H33" t="n">
-        <v>85494.084107</v>
+        <v>85508.831194</v>
       </c>
       <c r="I33" t="n">
-        <v>141057.306203</v>
+        <v>141114.283791</v>
       </c>
       <c r="J33" t="n">
         <v>164188.035231</v>
@@ -2958,19 +2958,19 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>27162.702669</v>
+        <v>27163.706756</v>
       </c>
       <c r="F34" t="n">
-        <v>69482.980396</v>
+        <v>69489.258821</v>
       </c>
       <c r="G34" t="n">
-        <v>175179.69262</v>
+        <v>175208.778329</v>
       </c>
       <c r="H34" t="n">
-        <v>413822.157993</v>
+        <v>413948.62118</v>
       </c>
       <c r="I34" t="n">
-        <v>856579.291184</v>
+        <v>857200.5095010001</v>
       </c>
       <c r="J34" t="n">
         <v>781461.382267</v>
@@ -3034,19 +3034,19 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>8399.357332</v>
+        <v>8399.557323000001</v>
       </c>
       <c r="F35" t="n">
-        <v>15044.612258</v>
+        <v>15045.491583</v>
       </c>
       <c r="G35" t="n">
-        <v>26718.473813</v>
+        <v>26721.270593</v>
       </c>
       <c r="H35" t="n">
-        <v>47892.997596</v>
+        <v>47902.002577</v>
       </c>
       <c r="I35" t="n">
-        <v>80548.48186699999</v>
+        <v>80584.20652399999</v>
       </c>
       <c r="J35" t="n">
         <v>87007.66338699999</v>
@@ -3110,19 +3110,19 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>176.820367</v>
+        <v>176.77054</v>
       </c>
       <c r="F36" t="n">
-        <v>255.260387</v>
+        <v>255.0744</v>
       </c>
       <c r="G36" t="n">
-        <v>332.797478</v>
+        <v>332.301456</v>
       </c>
       <c r="H36" t="n">
-        <v>463.621058</v>
+        <v>462.216429</v>
       </c>
       <c r="I36" t="n">
-        <v>660.8122</v>
+        <v>655.7888799999999</v>
       </c>
       <c r="J36" t="n">
         <v>5929.376647</v>
@@ -3186,19 +3186,19 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>7326.151812</v>
+        <v>7326.107426</v>
       </c>
       <c r="F37" t="n">
-        <v>9431.121408999999</v>
+        <v>9431.005342</v>
       </c>
       <c r="G37" t="n">
-        <v>12225.350359</v>
+        <v>12224.987541</v>
       </c>
       <c r="H37" t="n">
-        <v>17694.467052</v>
+        <v>17693.174822</v>
       </c>
       <c r="I37" t="n">
-        <v>26243.368229</v>
+        <v>26238.031842</v>
       </c>
       <c r="J37" t="n">
         <v>43828.163984</v>
@@ -3262,19 +3262,19 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>35064.604559</v>
+        <v>35065.791477</v>
       </c>
       <c r="F38" t="n">
-        <v>52006.961045</v>
+        <v>52011.474995</v>
       </c>
       <c r="G38" t="n">
-        <v>75951.368628</v>
+        <v>75964.18324100001</v>
       </c>
       <c r="H38" t="n">
-        <v>124124.75961</v>
+        <v>124165.234064</v>
       </c>
       <c r="I38" t="n">
-        <v>208563.364459</v>
+        <v>208730.337204</v>
       </c>
       <c r="J38" t="n">
         <v>153504.657633</v>
@@ -3338,19 +3338,19 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>3713.582456</v>
+        <v>3713.620063</v>
       </c>
       <c r="F39" t="n">
-        <v>5237.900472</v>
+        <v>5238.038909</v>
       </c>
       <c r="G39" t="n">
-        <v>7709.738499</v>
+        <v>7710.071414</v>
       </c>
       <c r="H39" t="n">
-        <v>12760.86977</v>
+        <v>12761.673454</v>
       </c>
       <c r="I39" t="n">
-        <v>21785.718711</v>
+        <v>21788.096826</v>
       </c>
       <c r="J39" t="n">
         <v>34842.927536</v>
@@ -3414,19 +3414,19 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>567.42921</v>
+        <v>567.428692</v>
       </c>
       <c r="F40" t="n">
-        <v>842.160977</v>
+        <v>842.158548</v>
       </c>
       <c r="G40" t="n">
-        <v>1250.10362</v>
+        <v>1250.081753</v>
       </c>
       <c r="H40" t="n">
-        <v>2011.665174</v>
+        <v>2011.545817</v>
       </c>
       <c r="I40" t="n">
-        <v>3308.807429</v>
+        <v>3308.158972</v>
       </c>
       <c r="J40" t="n">
         <v>6154.358516</v>
@@ -3490,19 +3490,19 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>667.90192</v>
+        <v>667.86071</v>
       </c>
       <c r="F41" t="n">
-        <v>1090.534649</v>
+        <v>1090.356525</v>
       </c>
       <c r="G41" t="n">
-        <v>1662.625438</v>
+        <v>1662.042628</v>
       </c>
       <c r="H41" t="n">
-        <v>2713.67982</v>
+        <v>2711.650831</v>
       </c>
       <c r="I41" t="n">
-        <v>4373.859341</v>
+        <v>4365.334316</v>
       </c>
       <c r="J41" t="n">
         <v>16409.643747</v>
@@ -3566,19 +3566,19 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>3941.605056</v>
+        <v>3941.234155</v>
       </c>
       <c r="F42" t="n">
-        <v>5302.09369</v>
+        <v>5300.854529</v>
       </c>
       <c r="G42" t="n">
-        <v>6815.263344</v>
+        <v>6812.054151</v>
       </c>
       <c r="H42" t="n">
-        <v>9625.821379000001</v>
+        <v>9616.654372999999</v>
       </c>
       <c r="I42" t="n">
-        <v>14154.744656</v>
+        <v>14120.797946</v>
       </c>
       <c r="J42" t="n">
         <v>55657.455196</v>
@@ -3642,19 +3642,19 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1654.183275</v>
+        <v>1654.236147</v>
       </c>
       <c r="F43" t="n">
-        <v>3324.56196</v>
+        <v>3324.825954</v>
       </c>
       <c r="G43" t="n">
-        <v>6228.287957</v>
+        <v>6229.216658</v>
       </c>
       <c r="H43" t="n">
-        <v>11848.757485</v>
+        <v>11852.079476</v>
       </c>
       <c r="I43" t="n">
-        <v>21807.048975</v>
+        <v>21821.777891</v>
       </c>
       <c r="J43" t="n">
         <v>20530.361647</v>
@@ -3718,19 +3718,19 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>7732.487137</v>
+        <v>7732.501192</v>
       </c>
       <c r="F44" t="n">
-        <v>12715.595018</v>
+        <v>12715.629568</v>
       </c>
       <c r="G44" t="n">
-        <v>19967.177128</v>
+        <v>19967.04443</v>
       </c>
       <c r="H44" t="n">
-        <v>34609.54254</v>
+        <v>34608.134511</v>
       </c>
       <c r="I44" t="n">
-        <v>61387.744666</v>
+        <v>61377.998505</v>
       </c>
       <c r="J44" t="n">
         <v>120863.573531</v>
@@ -3794,19 +3794,19 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>4607.658088</v>
+        <v>4607.770233</v>
       </c>
       <c r="F45" t="n">
-        <v>6941.579825</v>
+        <v>6942.011226</v>
       </c>
       <c r="G45" t="n">
-        <v>10223.406737</v>
+        <v>10224.608989</v>
       </c>
       <c r="H45" t="n">
-        <v>16391.06826</v>
+        <v>16394.690267</v>
       </c>
       <c r="I45" t="n">
-        <v>26252.227248</v>
+        <v>26266.246921</v>
       </c>
       <c r="J45" t="n">
         <v>25886.099123</v>
@@ -3870,19 +3870,19 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1611.094486</v>
+        <v>1610.993405</v>
       </c>
       <c r="F46" t="n">
-        <v>2724.107991</v>
+        <v>2723.657847</v>
       </c>
       <c r="G46" t="n">
-        <v>4554.507896</v>
+        <v>4552.873168</v>
       </c>
       <c r="H46" t="n">
-        <v>8077.349986</v>
+        <v>8071.115822</v>
       </c>
       <c r="I46" t="n">
-        <v>14365.017271</v>
+        <v>14335.764226</v>
       </c>
       <c r="J46" t="n">
         <v>62069.708785</v>
@@ -3946,19 +3946,19 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>136569.964298</v>
+        <v>136566.86542</v>
       </c>
       <c r="F47" t="n">
-        <v>230410.150434</v>
+        <v>230395.824185</v>
       </c>
       <c r="G47" t="n">
-        <v>360286.914963</v>
+        <v>360236.124287</v>
       </c>
       <c r="H47" t="n">
-        <v>604507.138295</v>
+        <v>604317.1185259999</v>
       </c>
       <c r="I47" t="n">
-        <v>1022849.080233</v>
+        <v>1021982.850298</v>
       </c>
       <c r="J47" t="n">
         <v>2755799.048378</v>
@@ -4022,19 +4022,19 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>12591.662601</v>
+        <v>12591.886058</v>
       </c>
       <c r="F48" t="n">
-        <v>19201.805597</v>
+        <v>19202.668466</v>
       </c>
       <c r="G48" t="n">
-        <v>28833.425544</v>
+        <v>28835.772171</v>
       </c>
       <c r="H48" t="n">
-        <v>46093.952267</v>
+        <v>46100.698412</v>
       </c>
       <c r="I48" t="n">
-        <v>73686.02388399999</v>
+        <v>73711.247527</v>
       </c>
       <c r="J48" t="n">
         <v>87865.690288</v>
@@ -4098,19 +4098,19 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2250.159954</v>
+        <v>2250.144121</v>
       </c>
       <c r="F49" t="n">
-        <v>3609.827068</v>
+        <v>3609.754161</v>
       </c>
       <c r="G49" t="n">
-        <v>5549.320295</v>
+        <v>5549.020291</v>
       </c>
       <c r="H49" t="n">
-        <v>9081.999033</v>
+        <v>9080.778708</v>
       </c>
       <c r="I49" t="n">
-        <v>14905.606417</v>
+        <v>14899.903015</v>
       </c>
       <c r="J49" t="n">
         <v>30278.431885</v>
@@ -4174,19 +4174,19 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>60.173065</v>
+        <v>60.168641</v>
       </c>
       <c r="F50" t="n">
-        <v>85.482821</v>
+        <v>85.466645</v>
       </c>
       <c r="G50" t="n">
-        <v>112.640692</v>
+        <v>112.596426</v>
       </c>
       <c r="H50" t="n">
-        <v>158.8834</v>
+        <v>158.754389</v>
       </c>
       <c r="I50" t="n">
-        <v>228.501225</v>
+        <v>228.027269</v>
       </c>
       <c r="J50" t="n">
         <v>808.424526</v>
@@ -4250,19 +4250,19 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>880.670002</v>
+        <v>880.328332</v>
       </c>
       <c r="F51" t="n">
-        <v>1261.222414</v>
+        <v>1259.983493</v>
       </c>
       <c r="G51" t="n">
-        <v>1801.655672</v>
+        <v>1798.042499</v>
       </c>
       <c r="H51" t="n">
-        <v>2818.376259</v>
+        <v>2806.848002</v>
       </c>
       <c r="I51" t="n">
-        <v>4594.465669</v>
+        <v>4547.093415</v>
       </c>
       <c r="J51" t="n">
         <v>61591.562824</v>
@@ -4326,19 +4326,19 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>910.16434</v>
+        <v>910.128514</v>
       </c>
       <c r="F52" t="n">
-        <v>1201.589354</v>
+        <v>1201.473529</v>
       </c>
       <c r="G52" t="n">
-        <v>1564.121715</v>
+        <v>1563.810878</v>
       </c>
       <c r="H52" t="n">
-        <v>2281.364403</v>
+        <v>2280.417006</v>
       </c>
       <c r="I52" t="n">
-        <v>3526.757695</v>
+        <v>3522.938271</v>
       </c>
       <c r="J52" t="n">
         <v>10141.135104</v>
@@ -4478,19 +4478,19 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>872963.100824</v>
+        <v>872963.264688</v>
       </c>
       <c r="F54" t="n">
-        <v>953742.611419</v>
+        <v>953743.013627</v>
       </c>
       <c r="G54" t="n">
-        <v>1126147.40333</v>
+        <v>1126148.276109</v>
       </c>
       <c r="H54" t="n">
-        <v>1313590.343382</v>
+        <v>1313592.253497</v>
       </c>
       <c r="I54" t="n">
-        <v>1513323.088807</v>
+        <v>1513328.278369</v>
       </c>
       <c r="J54" t="n">
         <v>1779492.642436</v>
@@ -4554,19 +4554,19 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>155023.924776</v>
+        <v>155023.760912</v>
       </c>
       <c r="F55" t="n">
-        <v>157518.492851</v>
+        <v>157518.090643</v>
       </c>
       <c r="G55" t="n">
-        <v>176137.70997</v>
+        <v>176136.837191</v>
       </c>
       <c r="H55" t="n">
-        <v>197713.602418</v>
+        <v>197711.692303</v>
       </c>
       <c r="I55" t="n">
-        <v>221503.741993</v>
+        <v>221498.552431</v>
       </c>
       <c r="J55" t="n">
         <v>195289.268364</v>
@@ -4782,19 +4782,19 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>19797.9771</v>
+        <v>19800.770015</v>
       </c>
       <c r="F58" t="n">
-        <v>25927.870448</v>
+        <v>25937.153267</v>
       </c>
       <c r="G58" t="n">
-        <v>35032.716071</v>
+        <v>35057.988995</v>
       </c>
       <c r="H58" t="n">
-        <v>45630.626616</v>
+        <v>45696.525375</v>
       </c>
       <c r="I58" t="n">
-        <v>59622.289147</v>
+        <v>59835.079091</v>
       </c>
       <c r="J58" t="n">
         <v>25375.27405</v>
@@ -4858,19 +4858,19 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>18290.967505</v>
+        <v>18294.438782</v>
       </c>
       <c r="F59" t="n">
-        <v>25884.865407</v>
+        <v>25897.280645</v>
       </c>
       <c r="G59" t="n">
-        <v>37487.02072</v>
+        <v>37523.160641</v>
       </c>
       <c r="H59" t="n">
-        <v>50263.808401</v>
+        <v>50360.707237</v>
       </c>
       <c r="I59" t="n">
-        <v>66158.219259</v>
+        <v>66473.909312</v>
       </c>
       <c r="J59" t="n">
         <v>9180.994720999999</v>
@@ -4934,19 +4934,19 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>14988.03757</v>
+        <v>14990.456996</v>
       </c>
       <c r="F60" t="n">
-        <v>15951.17061</v>
+        <v>15957.680681</v>
       </c>
       <c r="G60" t="n">
-        <v>17857.184579</v>
+        <v>17871.828567</v>
       </c>
       <c r="H60" t="n">
-        <v>20686.518157</v>
+        <v>20720.429675</v>
       </c>
       <c r="I60" t="n">
-        <v>25509.565946</v>
+        <v>25612.942762</v>
       </c>
       <c r="J60" t="n">
         <v>7730.545845</v>
@@ -5010,19 +5010,19 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>38923.785389</v>
+        <v>38923.640837</v>
       </c>
       <c r="F61" t="n">
-        <v>52721.910988</v>
+        <v>52721.797969</v>
       </c>
       <c r="G61" t="n">
-        <v>70707.194552</v>
+        <v>70707.511186</v>
       </c>
       <c r="H61" t="n">
-        <v>90698.767997</v>
+        <v>90700.59606</v>
       </c>
       <c r="I61" t="n">
-        <v>117844.505749</v>
+        <v>117852.281296</v>
       </c>
       <c r="J61" t="n">
         <v>148438.34857</v>
@@ -5086,19 +5086,19 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>73060.082077</v>
+        <v>73054.332985</v>
       </c>
       <c r="F62" t="n">
-        <v>101448.191116</v>
+        <v>101429.276709</v>
       </c>
       <c r="G62" t="n">
-        <v>136155.6523</v>
+        <v>136106.81488</v>
       </c>
       <c r="H62" t="n">
-        <v>171258.626955</v>
+        <v>171139.721935</v>
       </c>
       <c r="I62" t="n">
-        <v>214925.007596</v>
+        <v>214567.343505</v>
       </c>
       <c r="J62" t="n">
         <v>339509.79383</v>
@@ -5162,19 +5162,19 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>64797.209437</v>
+        <v>64794.342694</v>
       </c>
       <c r="F63" t="n">
-        <v>89294.95114799999</v>
+        <v>89285.81717900001</v>
       </c>
       <c r="G63" t="n">
-        <v>119768.174307</v>
+        <v>119744.944942</v>
       </c>
       <c r="H63" t="n">
-        <v>155326.205111</v>
+        <v>155268.649183</v>
       </c>
       <c r="I63" t="n">
-        <v>205807.845155</v>
+        <v>205627.040878</v>
       </c>
       <c r="J63" t="n">
         <v>308899.464235</v>
@@ -5238,19 +5238,19 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>5715.285925</v>
+        <v>5716.33339</v>
       </c>
       <c r="F64" t="n">
-        <v>6731.808866</v>
+        <v>6734.926682</v>
       </c>
       <c r="G64" t="n">
-        <v>8440.036741</v>
+        <v>8447.892889999999</v>
       </c>
       <c r="H64" t="n">
-        <v>10481.990528</v>
+        <v>10501.500158</v>
       </c>
       <c r="I64" t="n">
-        <v>13381.053885</v>
+        <v>13442.68665</v>
       </c>
       <c r="J64" t="n">
         <v>2362.656645</v>
@@ -5314,19 +5314,19 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>42117.68008</v>
+        <v>42111.023067</v>
       </c>
       <c r="F65" t="n">
-        <v>62399.281814</v>
+        <v>62375.352287</v>
       </c>
       <c r="G65" t="n">
-        <v>91900.90526</v>
+        <v>91832.18804399999</v>
       </c>
       <c r="H65" t="n">
-        <v>127640.94592</v>
+        <v>127454.936018</v>
       </c>
       <c r="I65" t="n">
-        <v>178195.872162</v>
+        <v>177573.914032</v>
       </c>
       <c r="J65" t="n">
         <v>393042.25083</v>
@@ -5390,19 +5390,19 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>32560.67825</v>
+        <v>32562.782544</v>
       </c>
       <c r="F66" t="n">
-        <v>47860.248448</v>
+        <v>47868.324188</v>
       </c>
       <c r="G66" t="n">
-        <v>70597.763719</v>
+        <v>70622.219816</v>
       </c>
       <c r="H66" t="n">
-        <v>98641.102421</v>
+        <v>98710.34845200001</v>
       </c>
       <c r="I66" t="n">
-        <v>137879.279653</v>
+        <v>138119.7602</v>
       </c>
       <c r="J66" t="n">
         <v>126058.56854</v>
@@ -5466,19 +5466,19 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>3747.012245</v>
+        <v>3745.379469</v>
       </c>
       <c r="F67" t="n">
-        <v>5593.270958</v>
+        <v>5587.295558</v>
       </c>
       <c r="G67" t="n">
-        <v>8794.809321999999</v>
+        <v>8776.436845</v>
       </c>
       <c r="H67" t="n">
-        <v>13396.650792</v>
+        <v>13342.300125</v>
       </c>
       <c r="I67" t="n">
-        <v>20775.049237</v>
+        <v>20576.275292</v>
       </c>
       <c r="J67" t="n">
         <v>84026.17458799999</v>
@@ -5542,19 +5542,19 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>14841.410711</v>
+        <v>14840.864816</v>
       </c>
       <c r="F68" t="n">
-        <v>21289.207532</v>
+        <v>21287.454576</v>
       </c>
       <c r="G68" t="n">
-        <v>32248.42887</v>
+        <v>32243.641207</v>
       </c>
       <c r="H68" t="n">
-        <v>45637.566264</v>
+        <v>45625.166793</v>
       </c>
       <c r="I68" t="n">
-        <v>62295.771788</v>
+        <v>62256.683492</v>
       </c>
       <c r="J68" t="n">
         <v>88012.861599</v>
@@ -5618,19 +5618,19 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>9881.894867999999</v>
+        <v>9883.655484999999</v>
       </c>
       <c r="F69" t="n">
-        <v>12928.423604</v>
+        <v>12934.248854</v>
       </c>
       <c r="G69" t="n">
-        <v>17082.354744</v>
+        <v>17097.828731</v>
       </c>
       <c r="H69" t="n">
-        <v>21613.838598</v>
+        <v>21652.98918</v>
       </c>
       <c r="I69" t="n">
-        <v>27469.087727</v>
+        <v>27592.177216</v>
       </c>
       <c r="J69" t="n">
         <v>5748.89486</v>
@@ -5694,19 +5694,19 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>16485.814058</v>
+        <v>16487.242793</v>
       </c>
       <c r="F70" t="n">
-        <v>23048.984727</v>
+        <v>23054.130732</v>
       </c>
       <c r="G70" t="n">
-        <v>33217.164453</v>
+        <v>33232.270279</v>
       </c>
       <c r="H70" t="n">
-        <v>46229.067255</v>
+        <v>46271.485527</v>
       </c>
       <c r="I70" t="n">
-        <v>65043.396374</v>
+        <v>65191.486936</v>
       </c>
       <c r="J70" t="n">
         <v>51235.364458</v>
@@ -5770,19 +5770,19 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>37056.467153</v>
+        <v>37057.83339</v>
       </c>
       <c r="F71" t="n">
-        <v>54393.087623</v>
+        <v>54398.52027</v>
       </c>
       <c r="G71" t="n">
-        <v>74375.32116799999</v>
+        <v>74390.777821</v>
       </c>
       <c r="H71" t="n">
-        <v>94581.531007</v>
+        <v>94621.50554699999</v>
       </c>
       <c r="I71" t="n">
-        <v>121922.852863</v>
+        <v>122050.767703</v>
       </c>
       <c r="J71" t="n">
         <v>124971.268003</v>
@@ -5846,19 +5846,19 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>21817.361261</v>
+        <v>21816.136166</v>
       </c>
       <c r="F72" t="n">
-        <v>27759.720208</v>
+        <v>27756.035967</v>
       </c>
       <c r="G72" t="n">
-        <v>36441.600288</v>
+        <v>36432.360085</v>
       </c>
       <c r="H72" t="n">
-        <v>46773.692539</v>
+        <v>46750.967872</v>
       </c>
       <c r="I72" t="n">
-        <v>61575.574358</v>
+        <v>61504.656332</v>
       </c>
       <c r="J72" t="n">
         <v>97562.346521</v>
@@ -5922,19 +5922,19 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>34446.670497</v>
+        <v>34447.986522</v>
       </c>
       <c r="F73" t="n">
-        <v>34853.345558</v>
+        <v>34856.792761</v>
       </c>
       <c r="G73" t="n">
-        <v>33688.532991</v>
+        <v>33695.202213</v>
       </c>
       <c r="H73" t="n">
-        <v>34157.655212</v>
+        <v>34171.10265</v>
       </c>
       <c r="I73" t="n">
-        <v>38424.572918</v>
+        <v>38461.716872</v>
       </c>
       <c r="J73" t="n">
         <v>36834.881231</v>
@@ -5998,19 +5998,19 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>5932.755876</v>
+        <v>5933.870048</v>
       </c>
       <c r="F74" t="n">
-        <v>8949.838444999999</v>
+        <v>8954.089174999999</v>
       </c>
       <c r="G74" t="n">
-        <v>12351.768317</v>
+        <v>12363.561257</v>
       </c>
       <c r="H74" t="n">
-        <v>15537.163628</v>
+        <v>15566.825613</v>
       </c>
       <c r="I74" t="n">
-        <v>19307.399581</v>
+        <v>19398.621832</v>
       </c>
       <c r="J74" t="n">
         <v>2778.206875</v>
@@ -6074,19 +6074,19 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>29631.738826</v>
+        <v>29631.327801</v>
       </c>
       <c r="F75" t="n">
-        <v>36715.899137</v>
+        <v>36714.446995</v>
       </c>
       <c r="G75" t="n">
-        <v>44349.259538</v>
+        <v>44344.808601</v>
       </c>
       <c r="H75" t="n">
-        <v>52291.049012</v>
+        <v>52278.924546</v>
       </c>
       <c r="I75" t="n">
-        <v>60740.325439</v>
+        <v>60703.510958</v>
       </c>
       <c r="J75" t="n">
         <v>92242.686739</v>
@@ -6150,19 +6150,19 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>93953.989397</v>
+        <v>93941.567866</v>
       </c>
       <c r="F76" t="n">
-        <v>118249.435211</v>
+        <v>118211.592255</v>
       </c>
       <c r="G76" t="n">
-        <v>115577.555665</v>
+        <v>115500.655137</v>
       </c>
       <c r="H76" t="n">
-        <v>116408.197708</v>
+        <v>116249.831691</v>
       </c>
       <c r="I76" t="n">
-        <v>128124.928665</v>
+        <v>127703.843443</v>
       </c>
       <c r="J76" t="n">
         <v>412587.015421</v>
@@ -6226,19 +6226,19 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>41160.10157</v>
+        <v>41159.465662</v>
       </c>
       <c r="F77" t="n">
-        <v>57850.6366</v>
+        <v>57848.437224</v>
       </c>
       <c r="G77" t="n">
-        <v>73056.24533600001</v>
+        <v>73049.42583199999</v>
       </c>
       <c r="H77" t="n">
-        <v>83341.41952900001</v>
+        <v>83323.012818</v>
       </c>
       <c r="I77" t="n">
-        <v>89651.983849</v>
+        <v>89598.200385</v>
       </c>
       <c r="J77" t="n">
         <v>127489.232628</v>
@@ -6302,19 +6302,19 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>349012.236637</v>
+        <v>349013.72978</v>
       </c>
       <c r="F78" t="n">
-        <v>373046.352904</v>
+        <v>373045.146805</v>
       </c>
       <c r="G78" t="n">
-        <v>377019.272366</v>
+        <v>377002.047421</v>
       </c>
       <c r="H78" t="n">
-        <v>397215.272621</v>
+        <v>397157.177955</v>
       </c>
       <c r="I78" t="n">
-        <v>443166.708809</v>
+        <v>442977.143103</v>
       </c>
       <c r="J78" t="n">
         <v>634771.353103</v>
@@ -6378,19 +6378,19 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>49470.170009</v>
+        <v>49472.115003</v>
       </c>
       <c r="F79" t="n">
-        <v>80968.49943500001</v>
+        <v>80975.79927600001</v>
       </c>
       <c r="G79" t="n">
-        <v>129620.267643</v>
+        <v>129640.222192</v>
       </c>
       <c r="H79" t="n">
-        <v>189766.309344</v>
+        <v>189817.217651</v>
       </c>
       <c r="I79" t="n">
-        <v>252823.715301</v>
+        <v>252976.653427</v>
       </c>
       <c r="J79" t="n">
         <v>208829.137654</v>
@@ -6454,19 +6454,19 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>20936.148943</v>
+        <v>20936.588912</v>
       </c>
       <c r="F80" t="n">
-        <v>22557.868369</v>
+        <v>22558.70391</v>
       </c>
       <c r="G80" t="n">
-        <v>24413.075863</v>
+        <v>24413.952832</v>
       </c>
       <c r="H80" t="n">
-        <v>28598.284406</v>
+        <v>28598.959001</v>
       </c>
       <c r="I80" t="n">
-        <v>35579.642943</v>
+        <v>35579.871796</v>
       </c>
       <c r="J80" t="n">
         <v>45120.251193</v>
@@ -6530,19 +6530,19 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>65151.909312</v>
+        <v>65154.902389</v>
       </c>
       <c r="F81" t="n">
-        <v>109009.430638</v>
+        <v>109020.949857</v>
       </c>
       <c r="G81" t="n">
-        <v>173601.704051</v>
+        <v>173633.352957</v>
       </c>
       <c r="H81" t="n">
-        <v>252257.623496</v>
+        <v>252338.72143</v>
       </c>
       <c r="I81" t="n">
-        <v>336577.721972</v>
+        <v>336824.480886</v>
       </c>
       <c r="J81" t="n">
         <v>250477.427228</v>
@@ -6606,19 +6606,19 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>85574.281518</v>
+        <v>85576.134533</v>
       </c>
       <c r="F82" t="n">
-        <v>106757.253617</v>
+        <v>106761.81281</v>
       </c>
       <c r="G82" t="n">
-        <v>125478.494836</v>
+        <v>125484.93669</v>
       </c>
       <c r="H82" t="n">
-        <v>148912.598504</v>
+        <v>148920.802554</v>
       </c>
       <c r="I82" t="n">
-        <v>177722.373692</v>
+        <v>177735.434798</v>
       </c>
       <c r="J82" t="n">
         <v>203372.331975</v>
@@ -6682,19 +6682,19 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>218025.358789</v>
+        <v>218030.103055</v>
       </c>
       <c r="F83" t="n">
-        <v>365541.598083</v>
+        <v>365560.084866</v>
       </c>
       <c r="G83" t="n">
-        <v>577756.421886</v>
+        <v>577802.895523</v>
       </c>
       <c r="H83" t="n">
-        <v>828074.526383</v>
+        <v>828180.633357</v>
       </c>
       <c r="I83" t="n">
-        <v>1077638.694875</v>
+        <v>1077926.956748</v>
       </c>
       <c r="J83" t="n">
         <v>1113301.569835</v>
@@ -6910,19 +6910,19 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>166057.9829</v>
+        <v>166058.126814</v>
       </c>
       <c r="F86" t="n">
-        <v>185542.065082</v>
+        <v>185542.47192</v>
       </c>
       <c r="G86" t="n">
-        <v>216361.696642</v>
+        <v>216362.653708</v>
       </c>
       <c r="H86" t="n">
-        <v>255301.455342</v>
+        <v>255303.716521</v>
       </c>
       <c r="I86" t="n">
-        <v>290252.44926</v>
+        <v>290258.817839</v>
       </c>
       <c r="J86" t="n">
         <v>155164.372231</v>
@@ -6986,19 +6986,19 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>15456.212138</v>
+        <v>15456.202494</v>
       </c>
       <c r="F87" t="n">
-        <v>19334.911909</v>
+        <v>19334.882432</v>
       </c>
       <c r="G87" t="n">
-        <v>25571.623289</v>
+        <v>25571.546908</v>
       </c>
       <c r="H87" t="n">
-        <v>33357.051453</v>
+        <v>33356.85484</v>
       </c>
       <c r="I87" t="n">
-        <v>41162.047049</v>
+        <v>41161.449976</v>
       </c>
       <c r="J87" t="n">
         <v>65137.889495</v>
@@ -7062,19 +7062,19 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>281533.354598</v>
+        <v>281533.47021</v>
       </c>
       <c r="F88" t="n">
-        <v>281902.353434</v>
+        <v>281902.649848</v>
       </c>
       <c r="G88" t="n">
-        <v>302598.444404</v>
+        <v>302599.092127</v>
       </c>
       <c r="H88" t="n">
-        <v>346122.102485</v>
+        <v>346123.590635</v>
       </c>
       <c r="I88" t="n">
-        <v>396565.933282</v>
+        <v>396570.149668</v>
       </c>
       <c r="J88" t="n">
         <v>338528.950749</v>
@@ -7138,19 +7138,19 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>34582.144284</v>
+        <v>34582.168487</v>
       </c>
       <c r="F89" t="n">
-        <v>36779.577556</v>
+        <v>36779.642852</v>
       </c>
       <c r="G89" t="n">
-        <v>42730.952892</v>
+        <v>42731.106279</v>
       </c>
       <c r="H89" t="n">
-        <v>50629.34411</v>
+        <v>50629.708288</v>
       </c>
       <c r="I89" t="n">
-        <v>57961.817985</v>
+        <v>57962.850218</v>
       </c>
       <c r="J89" t="n">
         <v>37446.51145</v>
@@ -7214,19 +7214,19 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>103484.720128</v>
+        <v>103484.644707</v>
       </c>
       <c r="F90" t="n">
-        <v>112034.401635</v>
+        <v>112034.201207</v>
       </c>
       <c r="G90" t="n">
-        <v>133140.720085</v>
+        <v>133140.25174</v>
       </c>
       <c r="H90" t="n">
-        <v>162082.281404</v>
+        <v>162081.154592</v>
       </c>
       <c r="I90" t="n">
-        <v>190448.028686</v>
+        <v>190444.77062</v>
       </c>
       <c r="J90" t="n">
         <v>301984.61686</v>
@@ -7290,19 +7290,19 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>14524.290737</v>
+        <v>14524.236921</v>
       </c>
       <c r="F91" t="n">
-        <v>16174.313508</v>
+        <v>16174.1647</v>
       </c>
       <c r="G91" t="n">
-        <v>18947.846271</v>
+        <v>18947.500303</v>
       </c>
       <c r="H91" t="n">
-        <v>22099.611486</v>
+        <v>22098.812531</v>
       </c>
       <c r="I91" t="n">
-        <v>24708.796806</v>
+        <v>24706.619047</v>
       </c>
       <c r="J91" t="n">
         <v>80794.764469</v>
@@ -7366,19 +7366,19 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>18862.821143</v>
+        <v>18862.806267</v>
       </c>
       <c r="F92" t="n">
-        <v>21177.819934</v>
+        <v>21177.778934</v>
       </c>
       <c r="G92" t="n">
-        <v>25639.980157</v>
+        <v>25639.882532</v>
       </c>
       <c r="H92" t="n">
-        <v>30728.677052</v>
+        <v>30728.445748</v>
       </c>
       <c r="I92" t="n">
-        <v>34892.345002</v>
+        <v>34891.698577</v>
       </c>
       <c r="J92" t="n">
         <v>54442.998169</v>
@@ -7442,19 +7442,19 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>4449.085645</v>
+        <v>4449.078915</v>
       </c>
       <c r="F93" t="n">
-        <v>5234.934172</v>
+        <v>5234.914592</v>
       </c>
       <c r="G93" t="n">
-        <v>6667.499706</v>
+        <v>6667.450372</v>
       </c>
       <c r="H93" t="n">
-        <v>8620.319191000001</v>
+        <v>8620.192913999999</v>
       </c>
       <c r="I93" t="n">
-        <v>10671.357825</v>
+        <v>10670.97427</v>
       </c>
       <c r="J93" t="n">
         <v>23152.054187</v>
@@ -7518,19 +7518,19 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>560114.877911</v>
+        <v>560114.751329</v>
       </c>
       <c r="F94" t="n">
-        <v>662068.461753</v>
+        <v>662068.109224</v>
       </c>
       <c r="G94" t="n">
-        <v>797613.878889</v>
+        <v>797613.071036</v>
       </c>
       <c r="H94" t="n">
-        <v>953540.358509</v>
+        <v>953538.476027</v>
       </c>
       <c r="I94" t="n">
-        <v>1088449.671215</v>
+        <v>1088444.374844</v>
       </c>
       <c r="J94" t="n">
         <v>1341588.669361</v>
@@ -7594,19 +7594,19 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>224663.702151</v>
+        <v>224663.713939</v>
       </c>
       <c r="F95" t="n">
-        <v>270436.066957</v>
+        <v>270436.11104</v>
       </c>
       <c r="G95" t="n">
-        <v>338865.410062</v>
+        <v>338865.537871</v>
       </c>
       <c r="H95" t="n">
-        <v>419396.191264</v>
+        <v>419396.526056</v>
       </c>
       <c r="I95" t="n">
-        <v>491113.883553</v>
+        <v>491114.859594</v>
       </c>
       <c r="J95" t="n">
         <v>522882.094482</v>
@@ -7670,19 +7670,19 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>90768.644023</v>
+        <v>90768.622732</v>
       </c>
       <c r="F96" t="n">
-        <v>95105.181279</v>
+        <v>95105.128215</v>
       </c>
       <c r="G96" t="n">
-        <v>102801.280218</v>
+        <v>102801.170105</v>
       </c>
       <c r="H96" t="n">
-        <v>116552.765425</v>
+        <v>116552.520872</v>
       </c>
       <c r="I96" t="n">
-        <v>131636.45866</v>
+        <v>131635.776966</v>
       </c>
       <c r="J96" t="n">
         <v>165286.49013</v>
@@ -7746,19 +7746,19 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>50494.264342</v>
+        <v>50494.277185</v>
       </c>
       <c r="F97" t="n">
-        <v>48841.271559</v>
+        <v>48841.303818</v>
       </c>
       <c r="G97" t="n">
-        <v>51237.833365</v>
+        <v>51237.903</v>
       </c>
       <c r="H97" t="n">
-        <v>57897.348258</v>
+        <v>57897.506957</v>
       </c>
       <c r="I97" t="n">
-        <v>66092.846659</v>
+        <v>66093.29436</v>
       </c>
       <c r="J97" t="n">
         <v>63151.704397</v>
@@ -7822,19 +7822,19 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>208543.330245</v>
+        <v>208542.774164</v>
       </c>
       <c r="F98" t="n">
-        <v>223678.460961</v>
+        <v>223676.979597</v>
       </c>
       <c r="G98" t="n">
-        <v>223407.075254</v>
+        <v>223404.078091</v>
       </c>
       <c r="H98" t="n">
-        <v>229436.05003</v>
+        <v>229429.790671</v>
       </c>
       <c r="I98" t="n">
-        <v>241297.961533</v>
+        <v>241281.381849</v>
       </c>
       <c r="J98" t="n">
         <v>273245.203614</v>
@@ -7898,19 +7898,19 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>231282.187738</v>
+        <v>231280.045573</v>
       </c>
       <c r="F99" t="n">
-        <v>286126.104723</v>
+        <v>286119.744242</v>
       </c>
       <c r="G99" t="n">
-        <v>334697.361614</v>
+        <v>334683.080372</v>
       </c>
       <c r="H99" t="n">
-        <v>388894.760993</v>
+        <v>388862.622177</v>
       </c>
       <c r="I99" t="n">
-        <v>446021.157353</v>
+        <v>445931.710864</v>
       </c>
       <c r="J99" t="n">
         <v>601177.8575789999</v>
@@ -7974,19 +7974,19 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>97567.43367899999</v>
+        <v>97566.154624</v>
       </c>
       <c r="F100" t="n">
-        <v>103640.874017</v>
+        <v>103637.477155</v>
       </c>
       <c r="G100" t="n">
-        <v>105174.503177</v>
+        <v>105167.619332</v>
       </c>
       <c r="H100" t="n">
-        <v>110382.595686</v>
+        <v>110368.198927</v>
       </c>
       <c r="I100" t="n">
-        <v>118708.393085</v>
+        <v>118670.164683</v>
       </c>
       <c r="J100" t="n">
         <v>170945.268469</v>
@@ -8050,19 +8050,19 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>231200.010335</v>
+        <v>231203.964431</v>
       </c>
       <c r="F101" t="n">
-        <v>263731.235152</v>
+        <v>263742.537432</v>
       </c>
       <c r="G101" t="n">
-        <v>283641.117678</v>
+        <v>283665.412958</v>
       </c>
       <c r="H101" t="n">
-        <v>308341.261546</v>
+        <v>308393.836079</v>
       </c>
       <c r="I101" t="n">
-        <v>336255.119272</v>
+        <v>336396.808318</v>
       </c>
       <c r="J101" t="n">
         <v>201019.994883</v>
@@ -8126,19 +8126,19 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>1937897.020652</v>
+        <v>1937914.726465</v>
       </c>
       <c r="F102" t="n">
-        <v>2344354.711847</v>
+        <v>2344409.189989</v>
       </c>
       <c r="G102" t="n">
-        <v>2703056.908445</v>
+        <v>2703184.331118</v>
       </c>
       <c r="H102" t="n">
-        <v>3129179.45133</v>
+        <v>3129476.24443</v>
       </c>
       <c r="I102" t="n">
-        <v>3599501.15525</v>
+        <v>3600350.280121</v>
       </c>
       <c r="J102" t="n">
         <v>3031843.839344</v>
@@ -8202,19 +8202,19 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>2165282.331554</v>
+        <v>2165295.089688</v>
       </c>
       <c r="F103" t="n">
-        <v>2238340.488495</v>
+        <v>2238373.273518</v>
       </c>
       <c r="G103" t="n">
-        <v>2177156.633799</v>
+        <v>2177219.601527</v>
       </c>
       <c r="H103" t="n">
-        <v>2195634.325582</v>
+        <v>2195759.317839</v>
       </c>
       <c r="I103" t="n">
-        <v>2282185.152943</v>
+        <v>2282503.296139</v>
       </c>
       <c r="J103" t="n">
         <v>2038673.036033</v>
@@ -8278,19 +8278,19 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>174708.710523</v>
+        <v>174706.2738</v>
       </c>
       <c r="F104" t="n">
-        <v>203673.446577</v>
+        <v>203666.508823</v>
       </c>
       <c r="G104" t="n">
-        <v>225679.818022</v>
+        <v>225664.819299</v>
       </c>
       <c r="H104" t="n">
-        <v>255795.797183</v>
+        <v>255762.627592</v>
       </c>
       <c r="I104" t="n">
-        <v>291366.784491</v>
+        <v>291275.026182</v>
       </c>
       <c r="J104" t="n">
         <v>431896.053479</v>
@@ -8354,19 +8354,19 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>95098.556809</v>
+        <v>95097.784396</v>
       </c>
       <c r="F105" t="n">
-        <v>111806.613805</v>
+        <v>111804.388972</v>
       </c>
       <c r="G105" t="n">
-        <v>126304.914192</v>
+        <v>126300.017593</v>
       </c>
       <c r="H105" t="n">
-        <v>143645.118756</v>
+        <v>143634.212653</v>
       </c>
       <c r="I105" t="n">
-        <v>162884.662959</v>
+        <v>162854.391328</v>
       </c>
       <c r="J105" t="n">
         <v>215720.692907</v>
@@ -8430,19 +8430,19 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>949218.91327</v>
+        <v>949206.6737470001</v>
       </c>
       <c r="F106" t="n">
-        <v>1156017.520252</v>
+        <v>1155981.459177</v>
       </c>
       <c r="G106" t="n">
-        <v>1354732.722175</v>
+        <v>1354651.309007</v>
       </c>
       <c r="H106" t="n">
-        <v>1577114.535249</v>
+        <v>1576930.816024</v>
       </c>
       <c r="I106" t="n">
-        <v>1808011.553778</v>
+        <v>1807501.03997</v>
       </c>
       <c r="J106" t="n">
         <v>2596806.853354</v>
@@ -8506,19 +8506,19 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>4510.629854</v>
+        <v>4509.4402</v>
       </c>
       <c r="F107" t="n">
-        <v>5812.754358</v>
+        <v>5808.973787</v>
       </c>
       <c r="G107" t="n">
-        <v>6730.551694</v>
+        <v>6721.923303</v>
       </c>
       <c r="H107" t="n">
-        <v>7821.00906</v>
+        <v>7801.375765</v>
       </c>
       <c r="I107" t="n">
-        <v>9324.544281</v>
+        <v>9268.909769</v>
       </c>
       <c r="J107" t="n">
         <v>77456.33207400001</v>
@@ -8582,19 +8582,19 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>371569.396402</v>
+        <v>371564.316351</v>
       </c>
       <c r="F108" t="n">
-        <v>430855.434242</v>
+        <v>430840.978234</v>
       </c>
       <c r="G108" t="n">
-        <v>465379.747274</v>
+        <v>465349.000557</v>
       </c>
       <c r="H108" t="n">
-        <v>508119.769441</v>
+        <v>508053.51306</v>
       </c>
       <c r="I108" t="n">
-        <v>557963.508123</v>
+        <v>557784.923667</v>
       </c>
       <c r="J108" t="n">
         <v>808532.41737</v>
@@ -8658,19 +8658,19 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>172855.743703</v>
+        <v>172856.179928</v>
       </c>
       <c r="F109" t="n">
-        <v>202435.5502</v>
+        <v>202436.920889</v>
       </c>
       <c r="G109" t="n">
-        <v>235387.995896</v>
+        <v>235391.475702</v>
       </c>
       <c r="H109" t="n">
-        <v>281985.08896</v>
+        <v>281994.047307</v>
       </c>
       <c r="I109" t="n">
-        <v>338938.788706</v>
+        <v>338967.013919</v>
       </c>
       <c r="J109" t="n">
         <v>358528.074171</v>
@@ -8734,19 +8734,19 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>545922.453121</v>
+        <v>545933.599006</v>
       </c>
       <c r="F110" t="n">
-        <v>671707.602997</v>
+        <v>671742.020153</v>
       </c>
       <c r="G110" t="n">
-        <v>785037.529366</v>
+        <v>785118.096634</v>
       </c>
       <c r="H110" t="n">
-        <v>910629.968709</v>
+        <v>910816.364879</v>
       </c>
       <c r="I110" t="n">
-        <v>1039133.008797</v>
+        <v>1039659.559288</v>
       </c>
       <c r="J110" t="n">
         <v>536212.691486</v>
@@ -8810,19 +8810,19 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>936059.7624379999</v>
+        <v>936057.146227</v>
       </c>
       <c r="F111" t="n">
-        <v>1123849.459472</v>
+        <v>1123842.323029</v>
       </c>
       <c r="G111" t="n">
-        <v>1268757.788354</v>
+        <v>1268743.130073</v>
       </c>
       <c r="H111" t="n">
-        <v>1435801.397434</v>
+        <v>1435770.503363</v>
       </c>
       <c r="I111" t="n">
-        <v>1624488.269754</v>
+        <v>1624405.655577</v>
       </c>
       <c r="J111" t="n">
         <v>1896582.806106</v>
@@ -8886,19 +8886,19 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1130411.219678</v>
+        <v>1130393.531399</v>
       </c>
       <c r="F112" t="n">
-        <v>1374631.314302</v>
+        <v>1374578.796403</v>
       </c>
       <c r="G112" t="n">
-        <v>1603133.13946</v>
+        <v>1603013.910835</v>
       </c>
       <c r="H112" t="n">
-        <v>1875933.309442</v>
+        <v>1875660.968635</v>
       </c>
       <c r="I112" t="n">
-        <v>2180815.029073</v>
+        <v>2180044.927726</v>
       </c>
       <c r="J112" t="n">
         <v>3379927.088531</v>
@@ -8962,58 +8962,58 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>119604.726081</v>
+        <v>119603.42546</v>
       </c>
       <c r="F113" t="n">
-        <v>123568.09511</v>
+        <v>123565.2041</v>
       </c>
       <c r="G113" t="n">
-        <v>112182.459282</v>
+        <v>112178.00819</v>
       </c>
       <c r="H113" t="n">
-        <v>116047.407125</v>
+        <v>116040.616766</v>
       </c>
       <c r="I113" t="n">
-        <v>126116.541655</v>
+        <v>126106.572596</v>
       </c>
       <c r="J113" t="n">
-        <v>140598.05744</v>
+        <v>140583.880667</v>
       </c>
       <c r="K113" t="n">
-        <v>155625.304893</v>
+        <v>155605.989569</v>
       </c>
       <c r="L113" t="n">
-        <v>169399.269236</v>
+        <v>169373.923524</v>
       </c>
       <c r="M113" t="n">
-        <v>180932.617588</v>
+        <v>180900.385053</v>
       </c>
       <c r="N113" t="n">
-        <v>190844.509352</v>
+        <v>190804.34065</v>
       </c>
       <c r="O113" t="n">
-        <v>198717.104574</v>
+        <v>198667.898594</v>
       </c>
       <c r="P113" t="n">
-        <v>202566.21581</v>
+        <v>202507.27788</v>
       </c>
       <c r="Q113" t="n">
-        <v>203364.476045</v>
+        <v>203294.82681</v>
       </c>
       <c r="R113" t="n">
-        <v>202462.603028</v>
+        <v>202380.568288</v>
       </c>
       <c r="S113" t="n">
-        <v>200522.206127</v>
+        <v>200425.233868</v>
       </c>
       <c r="T113" t="n">
-        <v>197216.590477</v>
+        <v>197101.213822</v>
       </c>
       <c r="U113" t="n">
-        <v>192539.465389</v>
+        <v>192400.557725</v>
       </c>
       <c r="V113" t="n">
-        <v>187407.905019</v>
+        <v>187236.280626</v>
       </c>
     </row>
     <row r="114">
@@ -9038,58 +9038,58 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>21230.245932</v>
+        <v>21230.24541</v>
       </c>
       <c r="F114" t="n">
-        <v>31392.181305</v>
+        <v>31392.235377</v>
       </c>
       <c r="G114" t="n">
-        <v>43297.094116</v>
+        <v>43297.286031</v>
       </c>
       <c r="H114" t="n">
-        <v>59485.050839</v>
+        <v>59485.492803</v>
       </c>
       <c r="I114" t="n">
-        <v>74700.34535600001</v>
+        <v>74701.134288</v>
       </c>
       <c r="J114" t="n">
-        <v>86729.33472699999</v>
+        <v>86730.539366</v>
       </c>
       <c r="K114" t="n">
-        <v>94215.36341799999</v>
+        <v>94217.012804</v>
       </c>
       <c r="L114" t="n">
-        <v>97937.44562899999</v>
+        <v>97939.539366</v>
       </c>
       <c r="M114" t="n">
-        <v>99100.289888</v>
+        <v>99102.820859</v>
       </c>
       <c r="N114" t="n">
-        <v>98857.137978</v>
+        <v>98860.107688</v>
       </c>
       <c r="O114" t="n">
-        <v>97604.947356</v>
+        <v>97608.360521</v>
       </c>
       <c r="P114" t="n">
-        <v>94697.57023100001</v>
+        <v>94701.422836</v>
       </c>
       <c r="Q114" t="n">
-        <v>90819.913724</v>
+        <v>90824.240513</v>
       </c>
       <c r="R114" t="n">
-        <v>86549.83343699999</v>
+        <v>86554.70342000001</v>
       </c>
       <c r="S114" t="n">
-        <v>82123.79859799999</v>
+        <v>82129.312105</v>
       </c>
       <c r="T114" t="n">
-        <v>77466.14980299999</v>
+        <v>77472.43161100001</v>
       </c>
       <c r="U114" t="n">
-        <v>72681.85111800001</v>
+        <v>72689.07840699999</v>
       </c>
       <c r="V114" t="n">
-        <v>68176.633426</v>
+        <v>68185.17277999999</v>
       </c>
     </row>
     <row r="115">
@@ -9114,58 +9114,58 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>568623.661987</v>
+        <v>568624.9631310001</v>
       </c>
       <c r="F115" t="n">
-        <v>678733.042155</v>
+        <v>678735.879093</v>
       </c>
       <c r="G115" t="n">
-        <v>777762.483323</v>
+        <v>777766.742499</v>
       </c>
       <c r="H115" t="n">
-        <v>958500.7814569999</v>
+        <v>958507.129851</v>
       </c>
       <c r="I115" t="n">
-        <v>1155045.233409</v>
+        <v>1155054.413536</v>
       </c>
       <c r="J115" t="n">
-        <v>1347857.834253</v>
+        <v>1347870.806387</v>
       </c>
       <c r="K115" t="n">
-        <v>1511833.716609</v>
+        <v>1511851.382547</v>
       </c>
       <c r="L115" t="n">
-        <v>1650267.383485</v>
+        <v>1650290.63546</v>
       </c>
       <c r="M115" t="n">
-        <v>1768572.737524</v>
+        <v>1768602.439089</v>
       </c>
       <c r="N115" t="n">
-        <v>1878136.773671</v>
+        <v>1878173.972662</v>
       </c>
       <c r="O115" t="n">
-        <v>1972508.35607</v>
+        <v>1972554.148885</v>
       </c>
       <c r="P115" t="n">
-        <v>2028573.587259</v>
+        <v>2028628.672584</v>
       </c>
       <c r="Q115" t="n">
-        <v>2052685.53663</v>
+        <v>2052750.859077</v>
       </c>
       <c r="R115" t="n">
-        <v>2057554.931135</v>
+        <v>2057632.095891</v>
       </c>
       <c r="S115" t="n">
-        <v>2049352.715896</v>
+        <v>2049444.174647</v>
       </c>
       <c r="T115" t="n">
-        <v>2025871.79009</v>
+        <v>2025980.884938</v>
       </c>
       <c r="U115" t="n">
-        <v>1987946.324604</v>
+        <v>1988078.004979</v>
       </c>
       <c r="V115" t="n">
-        <v>1936480.747797</v>
+        <v>1936643.832836</v>
       </c>
     </row>
     <row r="116">
@@ -9190,19 +9190,19 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>21238.000822</v>
+        <v>21237.821737</v>
       </c>
       <c r="F116" t="n">
-        <v>22429.417345</v>
+        <v>22428.971814</v>
       </c>
       <c r="G116" t="n">
-        <v>26158.976516</v>
+        <v>26157.992562</v>
       </c>
       <c r="H116" t="n">
-        <v>30191.076802</v>
+        <v>30188.90592</v>
       </c>
       <c r="I116" t="n">
-        <v>33303.106837</v>
+        <v>33297.388434</v>
       </c>
       <c r="J116" t="n">
         <v>29893.019329</v>
@@ -9266,19 +9266,19 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>56304.783387</v>
+        <v>56304.19206</v>
       </c>
       <c r="F117" t="n">
-        <v>70880.87067</v>
+        <v>70878.932703</v>
       </c>
       <c r="G117" t="n">
-        <v>87648.86098500001</v>
+        <v>87644.138466</v>
       </c>
       <c r="H117" t="n">
-        <v>102964.110675</v>
+        <v>102953.309266</v>
       </c>
       <c r="I117" t="n">
-        <v>113472.680977</v>
+        <v>113444.017967</v>
       </c>
       <c r="J117" t="n">
         <v>90550.088195</v>
@@ -9342,19 +9342,19 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>40523.535158</v>
+        <v>40525.264983</v>
       </c>
       <c r="F118" t="n">
-        <v>40341.923159</v>
+        <v>40346.195712</v>
       </c>
       <c r="G118" t="n">
-        <v>44052.664234</v>
+        <v>44061.91203</v>
       </c>
       <c r="H118" t="n">
-        <v>48330.036656</v>
+        <v>48350.008393</v>
       </c>
       <c r="I118" t="n">
-        <v>51837.17205</v>
+        <v>51888.718909</v>
       </c>
       <c r="J118" t="n">
         <v>112104.696344</v>
@@ -9418,19 +9418,19 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>20345.844786</v>
+        <v>20345.954511</v>
       </c>
       <c r="F119" t="n">
-        <v>24505.378358</v>
+        <v>24505.657546</v>
       </c>
       <c r="G119" t="n">
-        <v>31835.290165</v>
+        <v>31835.912799</v>
       </c>
       <c r="H119" t="n">
-        <v>39876.512113</v>
+        <v>39877.88767</v>
       </c>
       <c r="I119" t="n">
-        <v>46720.722009</v>
+        <v>46724.344505</v>
       </c>
       <c r="J119" t="n">
         <v>57255.826328</v>
@@ -9494,19 +9494,19 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>10818.375347</v>
+        <v>10818.251207</v>
       </c>
       <c r="F120" t="n">
-        <v>11520.149087</v>
+        <v>11519.835</v>
       </c>
       <c r="G120" t="n">
-        <v>13574.593333</v>
+        <v>13573.887636</v>
       </c>
       <c r="H120" t="n">
-        <v>15857.918241</v>
+        <v>15856.335041</v>
       </c>
       <c r="I120" t="n">
-        <v>17726.687788</v>
+        <v>17722.449682</v>
       </c>
       <c r="J120" t="n">
         <v>14777.467559</v>
@@ -9570,19 +9570,19 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>135449.355788</v>
+        <v>135448.517114</v>
       </c>
       <c r="F121" t="n">
-        <v>161214.204629</v>
+        <v>161211.570016</v>
       </c>
       <c r="G121" t="n">
-        <v>207096.16649</v>
+        <v>207089.206252</v>
       </c>
       <c r="H121" t="n">
-        <v>253585.646991</v>
+        <v>253568.59713</v>
       </c>
       <c r="I121" t="n">
-        <v>286795.377182</v>
+        <v>286748.605256</v>
       </c>
       <c r="J121" t="n">
         <v>260909.319411</v>
@@ -9646,19 +9646,19 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>943266.6157120001</v>
+        <v>943266.509387</v>
       </c>
       <c r="F122" t="n">
-        <v>1009178.271341</v>
+        <v>1009179.0518</v>
       </c>
       <c r="G122" t="n">
-        <v>1198715.881648</v>
+        <v>1198719.383625</v>
       </c>
       <c r="H122" t="n">
-        <v>1415802.350991</v>
+        <v>1415812.60905</v>
       </c>
       <c r="I122" t="n">
-        <v>1606456.187627</v>
+        <v>1606486.409717</v>
       </c>
       <c r="J122" t="n">
         <v>1838234.270305</v>
@@ -9722,19 +9722,19 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>65554.43865</v>
+        <v>65611.17419799999</v>
       </c>
       <c r="F123" t="n">
-        <v>84382.00131000001</v>
+        <v>84552.09628300001</v>
       </c>
       <c r="G123" t="n">
-        <v>94235.96542199999</v>
+        <v>94586.29723900001</v>
       </c>
       <c r="H123" t="n">
-        <v>104565.211342</v>
+        <v>105276.316882</v>
       </c>
       <c r="I123" t="n">
-        <v>113783.838955</v>
+        <v>115465.006312</v>
       </c>
       <c r="J123" t="n">
         <v>41380.791877</v>
@@ -9798,19 +9798,19 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>501439.154316</v>
+        <v>501646.856651</v>
       </c>
       <c r="F124" t="n">
-        <v>641081.962121</v>
+        <v>641691.833969</v>
       </c>
       <c r="G124" t="n">
-        <v>703000.528531</v>
+        <v>704205.503242</v>
       </c>
       <c r="H124" t="n">
-        <v>768617.478427</v>
+        <v>770953.903845</v>
       </c>
       <c r="I124" t="n">
-        <v>836984.525185</v>
+        <v>842227.193759</v>
       </c>
       <c r="J124" t="n">
         <v>661313.645211</v>
@@ -9874,19 +9874,19 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>233225.251033</v>
+        <v>232960.813151</v>
       </c>
       <c r="F125" t="n">
-        <v>278850.37588</v>
+        <v>278070.409059</v>
       </c>
       <c r="G125" t="n">
-        <v>285705.330555</v>
+        <v>284150.024028</v>
       </c>
       <c r="H125" t="n">
-        <v>304154.637549</v>
+        <v>301107.106591</v>
       </c>
       <c r="I125" t="n">
-        <v>350794.764608</v>
+        <v>343870.928677</v>
       </c>
       <c r="J125" t="n">
         <v>722672.45715</v>
@@ -10254,19 +10254,19 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>449014.813319</v>
+        <v>449019.313157</v>
       </c>
       <c r="F130" t="n">
-        <v>520792.249345</v>
+        <v>520803.455078</v>
       </c>
       <c r="G130" t="n">
-        <v>669039.522407</v>
+        <v>669062.506141</v>
       </c>
       <c r="H130" t="n">
-        <v>864698.559409</v>
+        <v>864745.224541</v>
       </c>
       <c r="I130" t="n">
-        <v>1109063.823139</v>
+        <v>1109185.872107</v>
       </c>
       <c r="J130" t="n">
         <v>1511420.181404</v>
@@ -10330,19 +10330,19 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>100353.665034</v>
+        <v>100352.142386</v>
       </c>
       <c r="F131" t="n">
-        <v>127938.334281</v>
+        <v>127933.09257</v>
       </c>
       <c r="G131" t="n">
-        <v>162141.4727</v>
+        <v>162127.15846</v>
       </c>
       <c r="H131" t="n">
-        <v>202293.36042</v>
+        <v>202255.834259</v>
       </c>
       <c r="I131" t="n">
-        <v>251586.641344</v>
+        <v>251468.641564</v>
       </c>
       <c r="J131" t="n">
         <v>145710.796555</v>
@@ -10406,19 +10406,19 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>989180.588094</v>
+        <v>989189.082792</v>
       </c>
       <c r="F132" t="n">
-        <v>1041392.677922</v>
+        <v>1041411.618051</v>
       </c>
       <c r="G132" t="n">
-        <v>1176360.781466</v>
+        <v>1176395.008837</v>
       </c>
       <c r="H132" t="n">
-        <v>1340397.787293</v>
+        <v>1340459.962167</v>
       </c>
       <c r="I132" t="n">
-        <v>1572746.424917</v>
+        <v>1572896.251383</v>
       </c>
       <c r="J132" t="n">
         <v>2022370.807774</v>
@@ -10482,19 +10482,19 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>242330.742346</v>
+        <v>242333.682968</v>
       </c>
       <c r="F133" t="n">
-        <v>386943.33466</v>
+        <v>386952.187935</v>
       </c>
       <c r="G133" t="n">
-        <v>632783.15178</v>
+        <v>632803.16613</v>
       </c>
       <c r="H133" t="n">
-        <v>917067.46348</v>
+        <v>917107.606618</v>
       </c>
       <c r="I133" t="n">
-        <v>1204698.255375</v>
+        <v>1204798.432212</v>
       </c>
       <c r="J133" t="n">
         <v>1579308.371165</v>
@@ -10558,19 +10558,19 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>226363.879103</v>
+        <v>226364.696491</v>
       </c>
       <c r="F134" t="n">
-        <v>220704.805577</v>
+        <v>220706.398903</v>
       </c>
       <c r="G134" t="n">
-        <v>240289.273464</v>
+        <v>240291.519574</v>
       </c>
       <c r="H134" t="n">
-        <v>274950.716688</v>
+        <v>274953.418245</v>
       </c>
       <c r="I134" t="n">
-        <v>328269.145644</v>
+        <v>328272.756062</v>
       </c>
       <c r="J134" t="n">
         <v>393651.145515</v>
@@ -10634,19 +10634,19 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>66985.732882</v>
+        <v>66985.42286599999</v>
       </c>
       <c r="F135" t="n">
-        <v>89309.762176</v>
+        <v>89308.364424</v>
       </c>
       <c r="G135" t="n">
-        <v>129725.532682</v>
+        <v>129720.290287</v>
       </c>
       <c r="H135" t="n">
-        <v>180341.969236</v>
+        <v>180324.960849</v>
       </c>
       <c r="I135" t="n">
-        <v>240829.62306</v>
+        <v>240769.131755</v>
       </c>
       <c r="J135" t="n">
         <v>216806.205412</v>
@@ -10710,19 +10710,19 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>240609.549522</v>
+        <v>240606.910734</v>
       </c>
       <c r="F136" t="n">
-        <v>236686.861944</v>
+        <v>236679.922647</v>
       </c>
       <c r="G136" t="n">
-        <v>238772.367277</v>
+        <v>238757.373059</v>
       </c>
       <c r="H136" t="n">
-        <v>245151.683655</v>
+        <v>245119.602458</v>
       </c>
       <c r="I136" t="n">
-        <v>270096.708469</v>
+        <v>270007.971236</v>
       </c>
       <c r="J136" t="n">
         <v>195038.256255</v>
@@ -10786,19 +10786,19 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>65723.925583</v>
+        <v>65724.67513600001</v>
       </c>
       <c r="F137" t="n">
-        <v>71181.165979</v>
+        <v>71182.921762</v>
       </c>
       <c r="G137" t="n">
-        <v>79889.63584</v>
+        <v>79892.98349</v>
       </c>
       <c r="H137" t="n">
-        <v>90451.979053</v>
+        <v>90458.466042</v>
       </c>
       <c r="I137" t="n">
-        <v>104848.512857</v>
+        <v>104865.008744</v>
       </c>
       <c r="J137" t="n">
         <v>139867.133676</v>
@@ -10862,19 +10862,19 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>115439.109002</v>
+        <v>115438.031948</v>
       </c>
       <c r="F138" t="n">
-        <v>120980.041772</v>
+        <v>120976.914483</v>
       </c>
       <c r="G138" t="n">
-        <v>137210.197871</v>
+        <v>137202.28876</v>
       </c>
       <c r="H138" t="n">
-        <v>154465.075903</v>
+        <v>154445.992812</v>
       </c>
       <c r="I138" t="n">
-        <v>173593.429443</v>
+        <v>173539.001633</v>
       </c>
       <c r="J138" t="n">
         <v>124804.680926</v>
@@ -10938,19 +10938,19 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>146178.337065</v>
+        <v>146174.643738</v>
       </c>
       <c r="F139" t="n">
-        <v>166054.056016</v>
+        <v>166043.17815</v>
       </c>
       <c r="G139" t="n">
-        <v>210559.253906</v>
+        <v>210530.438203</v>
       </c>
       <c r="H139" t="n">
-        <v>269514.607367</v>
+        <v>269438.656093</v>
       </c>
       <c r="I139" t="n">
-        <v>340906.161832</v>
+        <v>340665.311795</v>
       </c>
       <c r="J139" t="n">
         <v>88182.207908</v>
@@ -11014,19 +11014,19 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>1269411.895271</v>
+        <v>1269396.824965</v>
       </c>
       <c r="F140" t="n">
-        <v>1240427.727184</v>
+        <v>1240388.52958</v>
       </c>
       <c r="G140" t="n">
-        <v>1354409.640789</v>
+        <v>1354317.026809</v>
       </c>
       <c r="H140" t="n">
-        <v>1556120.738352</v>
+        <v>1555895.426191</v>
       </c>
       <c r="I140" t="n">
-        <v>1864165.070197</v>
+        <v>1863478.973749</v>
       </c>
       <c r="J140" t="n">
         <v>1309602.444595</v>
@@ -11090,19 +11090,19 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>70094.771593</v>
+        <v>70097.51742400001</v>
       </c>
       <c r="F141" t="n">
-        <v>83930.62128599999</v>
+        <v>83938.325304</v>
       </c>
       <c r="G141" t="n">
-        <v>109824.068594</v>
+        <v>109842.772071</v>
       </c>
       <c r="H141" t="n">
-        <v>142087.057701</v>
+        <v>142132.118533</v>
       </c>
       <c r="I141" t="n">
-        <v>183540.328198</v>
+        <v>183675.204859</v>
       </c>
       <c r="J141" t="n">
         <v>407948.377524</v>
@@ -11166,19 +11166,19 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>20383.608186</v>
+        <v>20387.672393</v>
       </c>
       <c r="F142" t="n">
-        <v>36271.961959</v>
+        <v>36288.691213</v>
       </c>
       <c r="G142" t="n">
-        <v>74001.246925</v>
+        <v>74063.613879</v>
       </c>
       <c r="H142" t="n">
-        <v>131245.543143</v>
+        <v>131449.27289</v>
       </c>
       <c r="I142" t="n">
-        <v>205907.268225</v>
+        <v>206628.835601</v>
       </c>
       <c r="J142" t="n">
         <v>1286551.50299</v>
@@ -11470,19 +11470,19 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>4255.859617</v>
+        <v>4255.794058</v>
       </c>
       <c r="F146" t="n">
-        <v>4104.925094</v>
+        <v>4104.766036</v>
       </c>
       <c r="G146" t="n">
-        <v>4466.248302</v>
+        <v>4465.90083</v>
       </c>
       <c r="H146" t="n">
-        <v>5317.68966</v>
+        <v>5316.86551</v>
       </c>
       <c r="I146" t="n">
-        <v>6734.233751</v>
+        <v>6731.672374</v>
       </c>
       <c r="J146" t="n">
         <v>10179.268116</v>
@@ -11546,19 +11546,19 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>8331.68053</v>
+        <v>8331.523937</v>
       </c>
       <c r="F147" t="n">
-        <v>9105.028826</v>
+        <v>9104.600968000001</v>
       </c>
       <c r="G147" t="n">
-        <v>10673.607155</v>
+        <v>10672.60358</v>
       </c>
       <c r="H147" t="n">
-        <v>12777.668844</v>
+        <v>12775.273981</v>
       </c>
       <c r="I147" t="n">
-        <v>15874.963296</v>
+        <v>15867.643555</v>
       </c>
       <c r="J147" t="n">
         <v>24211.895595</v>
@@ -11622,19 +11622,19 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>468684.293653</v>
+        <v>468684.515805</v>
       </c>
       <c r="F148" t="n">
-        <v>544145.76563</v>
+        <v>544146.352546</v>
       </c>
       <c r="G148" t="n">
-        <v>695498.671263</v>
+        <v>695500.02231</v>
       </c>
       <c r="H148" t="n">
-        <v>889154.069596</v>
+        <v>889157.288609</v>
       </c>
       <c r="I148" t="n">
-        <v>1121794.487953</v>
+        <v>1121804.36907</v>
       </c>
       <c r="J148" t="n">
         <v>1357780.816188</v>
@@ -11698,19 +11698,19 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>31448.01878</v>
+        <v>31447.300108</v>
       </c>
       <c r="F149" t="n">
-        <v>36250.177158</v>
+        <v>36248.15283</v>
       </c>
       <c r="G149" t="n">
-        <v>46216.169856</v>
+        <v>46211.027044</v>
       </c>
       <c r="H149" t="n">
-        <v>60761.368991</v>
+        <v>60747.881264</v>
       </c>
       <c r="I149" t="n">
-        <v>79808.769673</v>
+        <v>79765.436024</v>
       </c>
       <c r="J149" t="n">
         <v>173980.764174</v>
@@ -11774,19 +11774,19 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>262311.257635</v>
+        <v>262311.901612</v>
       </c>
       <c r="F150" t="n">
-        <v>294180.983101</v>
+        <v>294182.858859</v>
       </c>
       <c r="G150" t="n">
-        <v>365955.542881</v>
+        <v>365959.484087</v>
       </c>
       <c r="H150" t="n">
-        <v>459314.115255</v>
+        <v>459321.039795</v>
       </c>
       <c r="I150" t="n">
-        <v>556069.744123</v>
+        <v>556080.559844</v>
       </c>
       <c r="J150" t="n">
         <v>646700.1779219999</v>
@@ -11850,19 +11850,19 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>90287.619177</v>
+        <v>90286.49172999999</v>
       </c>
       <c r="F151" t="n">
-        <v>109442.582743</v>
+        <v>109439.331441</v>
       </c>
       <c r="G151" t="n">
-        <v>145641.939424</v>
+        <v>145633.354895</v>
       </c>
       <c r="H151" t="n">
-        <v>191660.158007</v>
+        <v>191637.164473</v>
       </c>
       <c r="I151" t="n">
-        <v>239992.064797</v>
+        <v>239918.877913</v>
       </c>
       <c r="J151" t="n">
         <v>410141.91507</v>
@@ -11926,19 +11926,19 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>167482.973829</v>
+        <v>167478.355827</v>
       </c>
       <c r="F152" t="n">
-        <v>204474.392438</v>
+        <v>204460.860781</v>
       </c>
       <c r="G152" t="n">
-        <v>259614.205411</v>
+        <v>259580.196549</v>
       </c>
       <c r="H152" t="n">
-        <v>324026.050964</v>
+        <v>323941.057033</v>
       </c>
       <c r="I152" t="n">
-        <v>389301.719423</v>
+        <v>389048.960621</v>
       </c>
       <c r="J152" t="n">
         <v>829110.2290019999</v>
@@ -12002,19 +12002,19 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>193790.134042</v>
+        <v>193795.935159</v>
       </c>
       <c r="F153" t="n">
-        <v>226397.860869</v>
+        <v>226414.66888</v>
       </c>
       <c r="G153" t="n">
-        <v>301240.025464</v>
+        <v>301283.60416</v>
       </c>
       <c r="H153" t="n">
-        <v>410938.93211</v>
+        <v>411053.512579</v>
       </c>
       <c r="I153" t="n">
-        <v>541898.748059</v>
+        <v>542259.210432</v>
       </c>
       <c r="J153" t="n">
         <v>120808.205769</v>
@@ -12078,19 +12078,19 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>47755.256538</v>
+        <v>47755.275564</v>
       </c>
       <c r="F154" t="n">
-        <v>57076.14275</v>
+        <v>57076.266269</v>
       </c>
       <c r="G154" t="n">
-        <v>71202.585724</v>
+        <v>71202.802025</v>
       </c>
       <c r="H154" t="n">
-        <v>86459.10983299999</v>
+        <v>86459.080015</v>
       </c>
       <c r="I154" t="n">
-        <v>99747.78208600001</v>
+        <v>99745.783325</v>
       </c>
       <c r="J154" t="n">
         <v>116175.136222</v>
@@ -12154,19 +12154,19 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>64518.539743</v>
+        <v>64527.652703</v>
       </c>
       <c r="F155" t="n">
-        <v>99111.29534500001</v>
+        <v>99145.137571</v>
       </c>
       <c r="G155" t="n">
-        <v>158240.321525</v>
+        <v>158344.859751</v>
       </c>
       <c r="H155" t="n">
-        <v>245236.022644</v>
+        <v>245549.59548</v>
       </c>
       <c r="I155" t="n">
-        <v>367868.737395</v>
+        <v>368998.556079</v>
       </c>
       <c r="J155" t="n">
         <v>240390.058779</v>
@@ -12230,19 +12230,19 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>224971.029198</v>
+        <v>224974.050387</v>
       </c>
       <c r="F156" t="n">
-        <v>334809.101712</v>
+        <v>334818.248911</v>
       </c>
       <c r="G156" t="n">
-        <v>516495.654312</v>
+        <v>516517.922753</v>
       </c>
       <c r="H156" t="n">
-        <v>768435.108547</v>
+        <v>768487.483699</v>
       </c>
       <c r="I156" t="n">
-        <v>1101122.768827</v>
+        <v>1101274.499764</v>
       </c>
       <c r="J156" t="n">
         <v>1464787.62439</v>
@@ -12306,19 +12306,19 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>1448.062561</v>
+        <v>1447.500014</v>
       </c>
       <c r="F157" t="n">
-        <v>2658.141928</v>
+        <v>2655.646406</v>
       </c>
       <c r="G157" t="n">
-        <v>4636.505756</v>
+        <v>4628.022718</v>
       </c>
       <c r="H157" t="n">
-        <v>7160.646615</v>
+        <v>7135.083548</v>
       </c>
       <c r="I157" t="n">
-        <v>10287.171241</v>
+        <v>10199.975459</v>
       </c>
       <c r="J157" t="n">
         <v>34281.014316</v>
@@ -12382,19 +12382,19 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>50174.822565</v>
+        <v>50169.268735</v>
       </c>
       <c r="F158" t="n">
-        <v>63938.904587</v>
+        <v>63920.56114</v>
       </c>
       <c r="G158" t="n">
-        <v>84438.02443400001</v>
+        <v>84388.04502799999</v>
       </c>
       <c r="H158" t="n">
-        <v>112119.27393</v>
+        <v>111985.072905</v>
       </c>
       <c r="I158" t="n">
-        <v>151028.295788</v>
+        <v>150587.807287</v>
       </c>
       <c r="J158" t="n">
         <v>301879.788667</v>
@@ -12458,19 +12458,19 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>616.807127</v>
+        <v>616.6284010000001</v>
       </c>
       <c r="F159" t="n">
-        <v>863.021153</v>
+        <v>862.395263</v>
       </c>
       <c r="G159" t="n">
-        <v>1266.806537</v>
+        <v>1264.975579</v>
       </c>
       <c r="H159" t="n">
-        <v>1799.639381</v>
+        <v>1794.506859</v>
       </c>
       <c r="I159" t="n">
-        <v>2502.743407</v>
+        <v>2485.680068</v>
       </c>
       <c r="J159" t="n">
         <v>7223.02102</v>
@@ -12534,19 +12534,19 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>13161.893806</v>
+        <v>13156.05476</v>
       </c>
       <c r="F160" t="n">
-        <v>19603.158295</v>
+        <v>19581.63373</v>
       </c>
       <c r="G160" t="n">
-        <v>30742.996836</v>
+        <v>30676.48357</v>
       </c>
       <c r="H160" t="n">
-        <v>47781.985683</v>
+        <v>47580.934309</v>
       </c>
       <c r="I160" t="n">
-        <v>74839.053142</v>
+        <v>74102.251143</v>
       </c>
       <c r="J160" t="n">
         <v>301683.254628</v>
@@ -12686,19 +12686,19 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>14849.501548</v>
+        <v>14849.579678</v>
       </c>
       <c r="F162" t="n">
-        <v>12042.301498</v>
+        <v>12042.316646</v>
       </c>
       <c r="G162" t="n">
-        <v>10284.439169</v>
+        <v>10284.245395</v>
       </c>
       <c r="H162" t="n">
-        <v>10133.767347</v>
+        <v>10133.101833</v>
       </c>
       <c r="I162" t="n">
-        <v>10931.37176</v>
+        <v>10929.228271</v>
       </c>
       <c r="J162" t="n">
         <v>13750.445351</v>
@@ -12762,19 +12762,19 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>1503.794926</v>
+        <v>1503.519846</v>
       </c>
       <c r="F163" t="n">
-        <v>2003.273397</v>
+        <v>2002.384386</v>
       </c>
       <c r="G163" t="n">
-        <v>2806.099789</v>
+        <v>2803.705165</v>
       </c>
       <c r="H163" t="n">
-        <v>3873.951716</v>
+        <v>3867.608082</v>
       </c>
       <c r="I163" t="n">
-        <v>5121.95923</v>
+        <v>5102.356485</v>
       </c>
       <c r="J163" t="n">
         <v>18535.0474</v>
@@ -12838,19 +12838,19 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>16394.269972</v>
+        <v>16391.984395</v>
       </c>
       <c r="F164" t="n">
-        <v>24611.218184</v>
+        <v>24603.011685</v>
       </c>
       <c r="G164" t="n">
-        <v>37382.057666</v>
+        <v>37358.294192</v>
       </c>
       <c r="H164" t="n">
-        <v>55656.993851</v>
+        <v>55589.603367</v>
       </c>
       <c r="I164" t="n">
-        <v>79111.11408699999</v>
+        <v>78888.083356</v>
       </c>
       <c r="J164" t="n">
         <v>254151.439918</v>
@@ -12914,19 +12914,19 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>57620.018231</v>
+        <v>57622.710663</v>
       </c>
       <c r="F165" t="n">
-        <v>76192.339141</v>
+        <v>76200.899616</v>
       </c>
       <c r="G165" t="n">
-        <v>92121.990141</v>
+        <v>92141.744158</v>
       </c>
       <c r="H165" t="n">
-        <v>114598.796077</v>
+        <v>114646.10935</v>
       </c>
       <c r="I165" t="n">
-        <v>141972.706167</v>
+        <v>142114.251522</v>
       </c>
       <c r="J165" t="n">
         <v>84072.796735</v>
@@ -12990,19 +12990,19 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>57233.835739</v>
+        <v>57230.775375</v>
       </c>
       <c r="F166" t="n">
-        <v>70157.135278</v>
+        <v>70147.794263</v>
       </c>
       <c r="G166" t="n">
-        <v>86985.722842</v>
+        <v>86962.735128</v>
       </c>
       <c r="H166" t="n">
-        <v>110645.097946</v>
+        <v>110587.712765</v>
       </c>
       <c r="I166" t="n">
-        <v>137958.078626</v>
+        <v>137786.998127</v>
       </c>
       <c r="J166" t="n">
         <v>271421.81684</v>
@@ -13066,19 +13066,19 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>530662.337201</v>
+        <v>530676.923219</v>
       </c>
       <c r="F167" t="n">
-        <v>616683.278941</v>
+        <v>616722.362602</v>
       </c>
       <c r="G167" t="n">
-        <v>738588.096476</v>
+        <v>738674.732427</v>
       </c>
       <c r="H167" t="n">
-        <v>938129.976388</v>
+        <v>938338.19878</v>
       </c>
       <c r="I167" t="n">
-        <v>1189579.985192</v>
+        <v>1190212.892841</v>
       </c>
       <c r="J167" t="n">
         <v>1067198.985764</v>
@@ -13142,19 +13142,19 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>459.091373</v>
+        <v>458.975412</v>
       </c>
       <c r="F168" t="n">
-        <v>595.328967</v>
+        <v>594.960986</v>
       </c>
       <c r="G168" t="n">
-        <v>780.96446</v>
+        <v>780.023181</v>
       </c>
       <c r="H168" t="n">
-        <v>1056.689281</v>
+        <v>1054.229519</v>
       </c>
       <c r="I168" t="n">
-        <v>1427.617099</v>
+        <v>1419.884557</v>
       </c>
       <c r="J168" t="n">
         <v>6886.709938</v>
@@ -13218,19 +13218,19 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>291468.04291</v>
+        <v>291461.700828</v>
       </c>
       <c r="F169" t="n">
-        <v>374921.567381</v>
+        <v>374900.622578</v>
       </c>
       <c r="G169" t="n">
-        <v>487066.424202</v>
+        <v>487010.983219</v>
       </c>
       <c r="H169" t="n">
-        <v>671250.87801</v>
+        <v>671100.896433</v>
       </c>
       <c r="I169" t="n">
-        <v>923508.400303</v>
+        <v>923023.358795</v>
       </c>
       <c r="J169" t="n">
         <v>1556815.864541</v>
@@ -13294,19 +13294,19 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>12748.394128</v>
+        <v>12746.851261</v>
       </c>
       <c r="F170" t="n">
-        <v>19664.685295</v>
+        <v>19658.983796</v>
       </c>
       <c r="G170" t="n">
-        <v>29276.756506</v>
+        <v>29260.420287</v>
       </c>
       <c r="H170" t="n">
-        <v>42151.770586</v>
+        <v>42106.431875</v>
       </c>
       <c r="I170" t="n">
-        <v>57683.956138</v>
+        <v>57537.565395</v>
       </c>
       <c r="J170" t="n">
         <v>169708.420811</v>
@@ -13370,19 +13370,19 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>67370.898371</v>
+        <v>67362.404563</v>
       </c>
       <c r="F171" t="n">
-        <v>82946.95097400001</v>
+        <v>82921.211283</v>
       </c>
       <c r="G171" t="n">
-        <v>103460.321403</v>
+        <v>103397.304148</v>
       </c>
       <c r="H171" t="n">
-        <v>132828.56825</v>
+        <v>132671.096965</v>
       </c>
       <c r="I171" t="n">
-        <v>168329.744567</v>
+        <v>167857.498822</v>
       </c>
       <c r="J171" t="n">
         <v>498715.681764</v>
@@ -13446,19 +13446,19 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>178332.927432</v>
+        <v>178327.310282</v>
       </c>
       <c r="F172" t="n">
-        <v>203438.001102</v>
+        <v>203421.291122</v>
       </c>
       <c r="G172" t="n">
-        <v>225257.397452</v>
+        <v>225218.523802</v>
       </c>
       <c r="H172" t="n">
-        <v>257525.151518</v>
+        <v>257433.512883</v>
       </c>
       <c r="I172" t="n">
-        <v>298494.191131</v>
+        <v>298230.99614</v>
       </c>
       <c r="J172" t="n">
         <v>502464.095151</v>
@@ -13522,19 +13522,19 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>1011.893251</v>
+        <v>1011.824794</v>
       </c>
       <c r="F173" t="n">
-        <v>1545.040843</v>
+        <v>1544.789973</v>
       </c>
       <c r="G173" t="n">
-        <v>2285.790045</v>
+        <v>2285.073706</v>
       </c>
       <c r="H173" t="n">
-        <v>3272.788368</v>
+        <v>3270.803119</v>
       </c>
       <c r="I173" t="n">
-        <v>4496.472077</v>
+        <v>4490.007109</v>
       </c>
       <c r="J173" t="n">
         <v>10184.349907</v>
@@ -13598,19 +13598,19 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>619168.7196599999</v>
+        <v>619167.1160489999</v>
       </c>
       <c r="F174" t="n">
-        <v>725200.495934</v>
+        <v>725193.321703</v>
       </c>
       <c r="G174" t="n">
-        <v>864188.431578</v>
+        <v>864166.240798</v>
       </c>
       <c r="H174" t="n">
-        <v>1076748.04793</v>
+        <v>1076686.659092</v>
       </c>
       <c r="I174" t="n">
-        <v>1331915.888993</v>
+        <v>1331728.212139</v>
       </c>
       <c r="J174" t="n">
         <v>1743394.775999</v>
@@ -13674,19 +13674,19 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>2096.431881</v>
+        <v>2096.396964</v>
       </c>
       <c r="F175" t="n">
-        <v>3773.834678</v>
+        <v>3773.700567</v>
       </c>
       <c r="G175" t="n">
-        <v>6576.484397</v>
+        <v>6576.082535</v>
       </c>
       <c r="H175" t="n">
-        <v>10850.382589</v>
+        <v>10849.232918</v>
       </c>
       <c r="I175" t="n">
-        <v>16566.356195</v>
+        <v>16562.641424</v>
       </c>
       <c r="J175" t="n">
         <v>25777.975073</v>
@@ -13750,19 +13750,19 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>179.675427</v>
+        <v>179.613449</v>
       </c>
       <c r="F176" t="n">
-        <v>198.857358</v>
+        <v>198.687782</v>
       </c>
       <c r="G176" t="n">
-        <v>231.435639</v>
+        <v>231.049122</v>
       </c>
       <c r="H176" t="n">
-        <v>287.221924</v>
+        <v>286.296631</v>
       </c>
       <c r="I176" t="n">
-        <v>366.492653</v>
+        <v>363.777326</v>
       </c>
       <c r="J176" t="n">
         <v>2110.132678</v>
@@ -13826,19 +13826,19 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>572357.869632</v>
+        <v>572370.251938</v>
       </c>
       <c r="F177" t="n">
-        <v>901895.875981</v>
+        <v>901944.602138</v>
       </c>
       <c r="G177" t="n">
-        <v>1347326.599078</v>
+        <v>1347469.786958</v>
       </c>
       <c r="H177" t="n">
-        <v>1893843.520667</v>
+        <v>1894237.099172</v>
       </c>
       <c r="I177" t="n">
-        <v>2443560.767701</v>
+        <v>2444792.74156</v>
       </c>
       <c r="J177" t="n">
         <v>2181368.863938</v>
@@ -13902,19 +13902,19 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>450.371807</v>
+        <v>450.22939</v>
       </c>
       <c r="F178" t="n">
-        <v>620.028495</v>
+        <v>619.551866</v>
       </c>
       <c r="G178" t="n">
-        <v>837.385882</v>
+        <v>836.135214</v>
       </c>
       <c r="H178" t="n">
-        <v>1146.398601</v>
+        <v>1143.100441</v>
       </c>
       <c r="I178" t="n">
-        <v>1562.999853</v>
+        <v>1552.607624</v>
       </c>
       <c r="J178" t="n">
         <v>8790.745585999999</v>
@@ -13978,19 +13978,19 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>312.026511</v>
+        <v>311.931895</v>
       </c>
       <c r="F179" t="n">
-        <v>376.996855</v>
+        <v>376.717306</v>
       </c>
       <c r="G179" t="n">
-        <v>474.491075</v>
+        <v>473.808363</v>
       </c>
       <c r="H179" t="n">
-        <v>611.974753</v>
+        <v>610.2825759999999</v>
       </c>
       <c r="I179" t="n">
-        <v>783.0040279999999</v>
+        <v>778.004307</v>
       </c>
       <c r="J179" t="n">
         <v>4045.958406</v>
@@ -14130,16 +14130,16 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>-4e-06</v>
+        <v>7e-06</v>
       </c>
       <c r="F181" t="n">
-        <v>4e-06</v>
+        <v>-6e-06</v>
       </c>
       <c r="G181" t="n">
-        <v>-5e-06</v>
+        <v>3e-06</v>
       </c>
       <c r="H181" t="n">
-        <v>-2e-06</v>
+        <v>3e-06</v>
       </c>
       <c r="I181" t="n">
         <v>3e-06</v>
@@ -14154,10 +14154,10 @@
         <v>4e-06</v>
       </c>
       <c r="M181" t="n">
-        <v>5e-06</v>
+        <v>4e-06</v>
       </c>
       <c r="N181" t="n">
-        <v>-3e-06</v>
+        <v>-2e-06</v>
       </c>
       <c r="O181" t="n">
         <v>-3e-06</v>
@@ -14166,16 +14166,16 @@
         <v>-0</v>
       </c>
       <c r="Q181" t="n">
+        <v>2e-06</v>
+      </c>
+      <c r="R181" t="n">
         <v>3e-06</v>
       </c>
-      <c r="R181" t="n">
+      <c r="S181" t="n">
         <v>2e-06</v>
       </c>
-      <c r="S181" t="n">
-        <v>1e-06</v>
-      </c>
       <c r="T181" t="n">
-        <v>-4e-06</v>
+        <v>-5e-06</v>
       </c>
       <c r="U181" t="n">
         <v>0</v>

</xml_diff>